<commit_message>
Update berita 2026-08-03 19:15 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-03.xlsx
+++ b/data/berita_antara_2026-08-03.xlsx
@@ -10631,28 +10631,28 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
+          <t>TNBTS tutup sebagian akses Bromo imbas kebakaran hutan Blok Batengan</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
+          <t>Mon, 03 Aug 2026 22:44:14 +0700</t>
         </is>
       </c>
       <c r="D309" t="inlineStr"/>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
+          <t>Balai Besar Taman Nasional Bromo Tengger Semeru (TNBTS) menutup sebagian akses wisata Gunung Bromo dari pintu masuk ...</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
+          <t>https://www.antaranews.com/berita/5678457/tnbts-tutup-sebagian-akses-bromo-imbas-kebakaran-hutan-blok-batengan</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001396577.jpg</t>
         </is>
       </c>
     </row>
@@ -10664,28 +10664,28 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
+          <t>KPK hentikan penyidikan enam kasus, termasuk kasus Sekjen DPR</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
+          <t>Mon, 03 Aug 2026 22:39:52 +0700</t>
         </is>
       </c>
       <c r="D310" t="inlineStr"/>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
+          <t>Komisi Pemberantasan Korupsi (KPK) menghentikan penyidikan enam kasus dugaan tindak pidana korupsi dengan menerbitkan ...</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
+          <t>https://www.antaranews.com/berita/5678453/kpk-hentikan-penyidikan-enam-kasus-termasuk-kasus-sekjen-dpr</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_8208.jpg</t>
         </is>
       </c>
     </row>
@@ -10697,61 +10697,61 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
+          <t>Sekjen Golkar hingga eks Menpora bakal beri materi di Mubes Kosgoro</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
+          <t>Mon, 03 Aug 2026 22:38:02 +0700</t>
         </is>
       </c>
       <c r="D311" t="inlineStr"/>
       <c r="E311" t="inlineStr">
         <is>
-          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
+          <t>Sekjen DPP Partai Golkar Muhammad Sarmuji hingga Menpora periode 2023-2025 Dito Ariotedjo akan memberikan materi dalam ...</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
+          <t>https://www.antaranews.com/berita/5678449/sekjen-golkar-hingga-eks-menpora-bakal-beri-materi-di-mubes-kosgoro</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000469031.jpg</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
+          <t>Briket ampas kopi inovasi dosen UTU Meulaboh kantongi sertifikat paten</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
+          <t>Mon, 03 Aug 2026 22:37:22 +0700</t>
         </is>
       </c>
       <c r="D312" t="inlineStr"/>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
+          <t>Inovasi pengolahan limbah ampas kopi menjadi briket bahan bakar padat yang efisien karya Dosen Fakultas Pertanian ...</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
+          <t>https://www.antaranews.com/berita/5678445/briket-ampas-kopi-inovasi-dosen-utu-meulaboh-kantongi-sertifikat-paten</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-briket-ampas-kopi-dosen-utu-meulaboh.jpeg</t>
         </is>
       </c>
     </row>
@@ -10763,193 +10763,193 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
+          <t>Indonesia-Thailand sepakat tingkatkan kerja sama pertahanan, keamanan</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
+          <t>Mon, 03 Aug 2026 22:35:28 +0700</t>
         </is>
       </c>
       <c r="D313" t="inlineStr"/>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
+          <t>Presiden Republik Indonesia Prabowo Subianto dan Perdana Menteri (PM) Thailand Anutin Charnvirakul sepakat untuk ...</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
+          <t>https://www.antaranews.com/berita/5678443/indonesia-thailand-sepakat-tingkatkan-kerja-sama-pertahanan-keamanan</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageXOTgJY.jpg</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
+          <t>Kepala BGN: Putusan MK perkuat Program Makan Bergizi Gratis</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
+          <t>Mon, 03 Aug 2026 22:32:37 +0700</t>
         </is>
       </c>
       <c r="D314" t="inlineStr"/>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono mengatakan putusan Mahkamah Konstitusi (MK) Nomor 40/PUU-XXIV/2026 yang ...</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
+          <t>https://www.antaranews.com/berita/5678436/kepala-bgn-putusan-mk-perkuat-program-makan-bergizi-gratis</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/189743.jpg</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
+          <t>Banjir kepung 15 titik di Kota Padang akibat cuaca ekstrem</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
+          <t>Mon, 03 Aug 2026 22:25:29 +0700</t>
         </is>
       </c>
       <c r="D315" t="inlineStr"/>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
+          <t>ANTARA - Hujan lebat disertai angin kencang memicu bencana di Kabupaten Agam, Kota Pariaman, dan Kota Padang, Sumatera ...</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
+          <t>https://www.antaranews.com/video/5678396/banjir-kepung-15-titik-di-kota-padang-akibat-cuaca-ekstrem</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BANJIR-KEPUNG-15-TITIK-DI-KOTA-PADANG-AKIBAT-CUACA-EKSTREM.jpg</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
+          <t>Erick ungkap strategi sebelum kembali ke bursa calon Ketum PSSI 2027</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
+          <t>Mon, 03 Aug 2026 22:22:41 +0700</t>
         </is>
       </c>
       <c r="D316" t="inlineStr"/>
       <c r="E316" t="inlineStr">
         <is>
-          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
+          <t>ANTARA - Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir tidak menutup kemungkinan untuk ...</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
+          <t>https://www.antaranews.com/video/5678327/erick-ungkap-strategi-sebelum-kembali-ke-bursa-calon-ketum-pssi-2027</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/ERICK-UNGKAP-STRATEGI-SEBELUM-KEMBALI-KE-BURSA-CALON-KETUM-PSSI-2027.jpg</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
+          <t>Daop 6 Yogyakarta tutup perlintasan tak terjaga Petak Sentolo–Rewulu</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
+          <t>Mon, 03 Aug 2026 21:28:06 +0700</t>
         </is>
       </c>
       <c r="D317" t="inlineStr"/>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
+          <t>PT Kereta Api Indonesia (Persero) Daerah Operasi 6 Yogyakarta terus berkolaborasi dengan pemerintah terkait, untuk ...</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
+          <t>https://www.antaranews.com/berita/5678331/daop-6-yogyakarta-tutup-perlintasan-tak-terjaga-petak-sentolo-rewulu</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029465.jpg</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
+          <t>Kementan usulkan telur masuk skema CPP demi lindungi peternak rakyat</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
+          <t>Mon, 03 Aug 2026 21:27:37 +0700</t>
         </is>
       </c>
       <c r="D318" t="inlineStr"/>
       <c r="E318" t="inlineStr">
         <is>
-          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
+          <t>Kementerian Pertanian (Kementan) mengusulkan komoditas telur ayam masuk dalam skema pengadaan Cadangan Pangan ...</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
+          <t>https://www.antaranews.com/berita/5678329/kementan-usulkan-telur-masuk-skema-cpp-demi-lindungi-peternak-rakyat</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/9C2BC3E9-1C7E-4159-8805-C378B9294E25.jpeg</t>
         </is>
       </c>
     </row>
@@ -10961,28 +10961,28 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
+          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
+          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
         </is>
       </c>
       <c r="D319" t="inlineStr"/>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
+          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
+          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
         </is>
       </c>
     </row>
@@ -10994,94 +10994,94 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
+          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
+          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
         </is>
       </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
-          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
+          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
+          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
+          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
+          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
         </is>
       </c>
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr">
         <is>
-          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
+          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
+          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
+          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
+          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
         </is>
       </c>
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
+          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
+          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
         </is>
       </c>
     </row>
@@ -11093,28 +11093,28 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
+          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
         </is>
       </c>
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
+          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
+          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
         </is>
       </c>
     </row>
@@ -11126,28 +11126,28 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
+          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
         </is>
       </c>
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
+          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
+          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
         </is>
       </c>
     </row>
@@ -11159,61 +11159,61 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
+          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
         </is>
       </c>
       <c r="D325" t="inlineStr"/>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
+          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
+          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
+          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
+          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
         </is>
       </c>
       <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
+          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
+          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
         </is>
       </c>
     </row>
@@ -11225,61 +11225,61 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
+          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
+          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
         </is>
       </c>
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
+          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
+          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
+          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
         </is>
       </c>
       <c r="D328" t="inlineStr"/>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
+          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
+          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11291,94 +11291,94 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
+          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
         </is>
       </c>
       <c r="D329" t="inlineStr"/>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
+          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
+          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
+          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
         </is>
       </c>
       <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
+          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
+          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
+          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
+          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
+          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
+          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
         </is>
       </c>
     </row>
@@ -11390,28 +11390,28 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Presiden Prabowo terima kunjungan PM Thailand di Istana Merdeka</t>
+          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:59:27 +0700</t>
+          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
       <c r="E332" t="inlineStr">
         <is>
-          <t>ANTARA - Presiden Prabowo Subianto menerima kunjungan resmi Perdana Menteri Thailand Anutin Charnvirakul di Istana ...</t>
+          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678461/presiden-prabowo-terima-kunjungan-pm-thailand-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRESIDEN-PRABOWO-TERIMA-KUNJUNGAN-PM-THAILAND-DI-ISTANA-MERDEKA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11423,28 +11423,28 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Basarnas jemput 66 korban KM Mutiara Sentosa II dari Masalembu</t>
+          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:58:38 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) mengerahkan satu unit kapal untuk menjemput 66 korban ...</t>
+          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678472/basarnas-jemput-66-korban-km-mutiara-sentosa-ii-dari-masalembu</t>
+          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BASARNAS-JEMPUT-66-KORBAN-KM-MUTIARA-SENTOSA-II-DARI-MASALEMBU.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
         </is>
       </c>
     </row>
@@ -11456,61 +11456,61 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Kementerian ATR/BPN telah terbitkan 124 ribu SK sertifikat rumah MBR</t>
+          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:56:36 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
         </is>
       </c>
       <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) menyatakan telah menerbitkan surat keputusan ...</t>
+          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678484/kementerian-atr-bpn-telah-terbitkan-124-ribu-sk-sertifikat-rumah-mbr</t>
+          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_224532.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Timnas Indonesia dibungkam Vietnam 0-3</t>
+          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:54:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
         </is>
       </c>
       <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Timnas Indonesia dibungkam Vietnam 0-3 di kandang pada laga lanjutan Grup A Piala AFF 2026 di Stadion Pakansari, Bogor, ...</t>
+          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678480/timnas-indonesia-dibungkam-vietnam-0-3</t>
+          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-21a.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
         </is>
       </c>
     </row>
@@ -11522,28 +11522,28 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Prabowo-PM Thailand perkuat kemitraan strategis ASEAN</t>
+          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:52:55 +0700</t>
+          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Presiden RI Prabowo Subianto dan Perdana Menteri (PM) Thailand Anutin Charnvirakul sepakat memperkuat kemitraan ...</t>
+          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678476/prabowo-pm-thailand-perkuat-kemitraan-strategis-asean</t>
+          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_F6F7E006D3CC-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
         </is>
       </c>
     </row>
@@ -11555,61 +11555,61 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Galaxy Tab S12 Ultra mejeng di Geekbench, hadir dengan Dimensity 9500</t>
+          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:48:03 +0700</t>
+          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Samsung Galaxy Tab S12 Ultra dalam seri perangkat Galaxy Tab S12 yang diperkirakan dirilis September 2026 muncul di ...</t>
+          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678469/galaxy-tab-s12-ultra-mejeng-di-geekbench-hadir-dengan-dimensity-9500</t>
+          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/InShot_20260803_215836626.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Menteri PKP tegaskan KUR Perumahan perkuat ekonomi keluarga</t>
+          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:47:11 +0700</t>
+          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
         </is>
       </c>
       <c r="D338" t="inlineStr"/>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Menteri Perumahan dan Kawasan Permukiman (PKP) Maruarar Sirait menegaskan bahwa Kredit Usaha Rakyat (KUR) Perumahan ...</t>
+          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678465/menteri-pkp-tegaskan-kur-perumahan-perkuat-ekonomi-keluarga</t>
+          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1321013.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
         </is>
       </c>
     </row>
@@ -11621,61 +11621,61 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>TNBTS tutup sebagian akses Bromo imbas kebakaran hutan Blok Batengan</t>
+          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:44:14 +0700</t>
+          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Balai Besar Taman Nasional Bromo Tengger Semeru (TNBTS) menutup sebagian akses wisata Gunung Bromo dari pintu masuk ...</t>
+          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678457/tnbts-tutup-sebagian-akses-bromo-imbas-kebakaran-hutan-blok-batengan</t>
+          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001396577.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>KPK hentikan penyidikan enam kasus, termasuk kasus Sekjen DPR</t>
+          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:39:52 +0700</t>
+          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Komisi Pemberantasan Korupsi (KPK) menghentikan penyidikan enam kasus dugaan tindak pidana korupsi dengan menerbitkan ...</t>
+          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678453/kpk-hentikan-penyidikan-enam-kasus-termasuk-kasus-sekjen-dpr</t>
+          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_8208.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
         </is>
       </c>
     </row>
@@ -11687,28 +11687,28 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Sekjen Golkar hingga eks Menpora bakal beri materi di Mubes Kosgoro</t>
+          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:38:02 +0700</t>
+          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Sekjen DPP Partai Golkar Muhammad Sarmuji hingga Menpora periode 2023-2025 Dito Ariotedjo akan memberikan materi dalam ...</t>
+          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678449/sekjen-golkar-hingga-eks-menpora-bakal-beri-materi-di-mubes-kosgoro</t>
+          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000469031.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
         </is>
       </c>
     </row>
@@ -11720,28 +11720,28 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Briket ampas kopi inovasi dosen UTU Meulaboh kantongi sertifikat paten</t>
+          <t>Presiden Prabowo terima kunjungan PM Thailand di Istana Merdeka</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:37:22 +0700</t>
+          <t>Mon, 03 Aug 2026 22:59:27 +0700</t>
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Inovasi pengolahan limbah ampas kopi menjadi briket bahan bakar padat yang efisien karya Dosen Fakultas Pertanian ...</t>
+          <t>ANTARA - Presiden Prabowo Subianto menerima kunjungan resmi Perdana Menteri Thailand Anutin Charnvirakul di Istana ...</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678445/briket-ampas-kopi-inovasi-dosen-utu-meulaboh-kantongi-sertifikat-paten</t>
+          <t>https://www.antaranews.com/video/5678461/presiden-prabowo-terima-kunjungan-pm-thailand-di-istana-merdeka</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-briket-ampas-kopi-dosen-utu-meulaboh.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRESIDEN-PRABOWO-TERIMA-KUNJUNGAN-PM-THAILAND-DI-ISTANA-MERDEKA.jpg</t>
         </is>
       </c>
     </row>
@@ -11753,28 +11753,28 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand sepakat tingkatkan kerja sama pertahanan, keamanan</t>
+          <t>Basarnas jemput 66 korban KM Mutiara Sentosa II dari Masalembu</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:35:28 +0700</t>
+          <t>Mon, 03 Aug 2026 22:58:38 +0700</t>
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Presiden Republik Indonesia Prabowo Subianto dan Perdana Menteri (PM) Thailand Anutin Charnvirakul sepakat untuk ...</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) mengerahkan satu unit kapal untuk menjemput 66 korban ...</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678443/indonesia-thailand-sepakat-tingkatkan-kerja-sama-pertahanan-keamanan</t>
+          <t>https://www.antaranews.com/video/5678472/basarnas-jemput-66-korban-km-mutiara-sentosa-ii-dari-masalembu</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageXOTgJY.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BASARNAS-JEMPUT-66-KORBAN-KM-MUTIARA-SENTOSA-II-DARI-MASALEMBU.jpg</t>
         </is>
       </c>
     </row>
@@ -11786,28 +11786,28 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Ekonom: Inflasi mereda, semester II jadi momentum jaga keseimbangan</t>
+          <t>Kementerian ATR/BPN telah terbitkan 124 ribu SK sertifikat rumah MBR</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:34:25 +0700</t>
+          <t>Mon, 03 Aug 2026 22:56:36 +0700</t>
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Kepala Ekonom Trimegah Sekuritas Indonesia Fakhrul Fulvian menilai semester II-2026 menjadi momentum untuk menjaga ...</t>
+          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) menyatakan telah menerbitkan surat keputusan ...</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678439/ekonom-inflasi-mereda-semester-ii-jadi-momentum-jaga-keseimbangan</t>
+          <t>https://www.antaranews.com/berita/5678484/kementerian-atr-bpn-telah-terbitkan-124-ribu-sk-sertifikat-rumah-mbr</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/01/21/IMG_2637.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_224532.jpg</t>
         </is>
       </c>
     </row>
@@ -11819,61 +11819,61 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Kepala BGN: Putusan MK perkuat Program Makan Bergizi Gratis</t>
+          <t>Timnas Indonesia dibungkam Vietnam 0-3</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:32:37 +0700</t>
+          <t>Mon, 03 Aug 2026 22:54:01 +0700</t>
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono mengatakan putusan Mahkamah Konstitusi (MK) Nomor 40/PUU-XXIV/2026 yang ...</t>
+          <t>Timnas Indonesia dibungkam Vietnam 0-3 di kandang pada laga lanjutan Grup A Piala AFF 2026 di Stadion Pakansari, Bogor, ...</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678436/kepala-bgn-putusan-mk-perkuat-program-makan-bergizi-gratis</t>
+          <t>https://www.antaranews.com/berita/5678480/timnas-indonesia-dibungkam-vietnam-0-3</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/189743.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-21a.jpg</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>photo, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Piala AFF 2026 : Indonesia takluk 0-3 dari Vietnam</t>
+          <t>Prabowo-PM Thailand perkuat kemitraan strategis ASEAN</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:26:45 +0700</t>
+          <t>Mon, 03 Aug 2026 22:52:55 +0700</t>
         </is>
       </c>
       <c r="D346" t="inlineStr"/>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Pelatih Timnas Indonesia Jhon Herdman memberikan arahan kepada anak didiknya saat melawan Timnas Vietnam pada ...</t>
+          <t>Presiden RI Prabowo Subianto dan Perdana Menteri (PM) Thailand Anutin Charnvirakul sepakat memperkuat kemitraan ...</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5678435/piala-aff-2026-indonesia-takluk-0-3-dari-vietnam</t>
+          <t>https://www.antaranews.com/berita/5678476/prabowo-pm-thailand-perkuat-kemitraan-strategis-asean</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-11b.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_F6F7E006D3CC-1.jpeg</t>
         </is>
       </c>
     </row>
@@ -11885,127 +11885,127 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Banjir kepung 15 titik di Kota Padang akibat cuaca ekstrem</t>
+          <t>Galaxy Tab S12 Ultra mejeng di Geekbench, hadir dengan Dimensity 9500</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:25:29 +0700</t>
+          <t>Mon, 03 Aug 2026 22:48:03 +0700</t>
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr">
         <is>
-          <t>ANTARA - Hujan lebat disertai angin kencang memicu bencana di Kabupaten Agam, Kota Pariaman, dan Kota Padang, Sumatera ...</t>
+          <t>Samsung Galaxy Tab S12 Ultra dalam seri perangkat Galaxy Tab S12 yang diperkirakan dirilis September 2026 muncul di ...</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678396/banjir-kepung-15-titik-di-kota-padang-akibat-cuaca-ekstrem</t>
+          <t>https://www.antaranews.com/berita/5678469/galaxy-tab-s12-ultra-mejeng-di-geekbench-hadir-dengan-dimensity-9500</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BANJIR-KEPUNG-15-TITIK-DI-KOTA-PADANG-AKIBAT-CUACA-EKSTREM.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/InShot_20260803_215836626.jpg</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Pemkab Aceh Tenggara batasi pembelian BBM untuk cegah penimbunan</t>
+          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:25:13 +0700</t>
+          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Pemerintah Kabupaten Aceh Tenggara bersama Forkopimda setempat saat ini telah melakukan pembatasan pembelian bahan ...</t>
+          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678431/pemkab-aceh-tenggara-batasi-pembelian-bbm-untuk-cegah-penimbunan</t>
+          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-Bupati-Aceh-Tenggara-HM-Salim-Fakhry.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>MTI dorong kemudahan transaksi nirsentuh di MRT Jakarta</t>
+          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:24:07 +0700</t>
+          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
         </is>
       </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr">
         <is>
-          <t>PT Mitra Transaksi Indonesia (MTI) atau YOKKE mendukung penerapan sistem pembayaran kartu nirsentuh berbasis Europay, ...</t>
+          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678427/mti-dorong-kemudahan-transaksi-nirsentuh-di-mrt-jakarta</t>
+          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.59.08.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Erick ungkap strategi sebelum kembali ke bursa calon Ketum PSSI 2027</t>
+          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:22:41 +0700</t>
+          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
         </is>
       </c>
       <c r="D350" t="inlineStr"/>
       <c r="E350" t="inlineStr">
         <is>
-          <t>ANTARA - Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir tidak menutup kemungkinan untuk ...</t>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678327/erick-ungkap-strategi-sebelum-kembali-ke-bursa-calon-ketum-pssi-2027</t>
+          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/ERICK-UNGKAP-STRATEGI-SEBELUM-KEMBALI-KE-BURSA-CALON-KETUM-PSSI-2027.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
         </is>
       </c>
     </row>
@@ -12017,94 +12017,94 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
+          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
+          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
         </is>
       </c>
       <c r="D351" t="inlineStr"/>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
+          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
+          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
+          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
+          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
         </is>
       </c>
       <c r="D352" t="inlineStr"/>
       <c r="E352" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
+          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
+          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
+          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
+          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
         </is>
       </c>
     </row>
@@ -12116,61 +12116,61 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
+          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
+          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
         </is>
       </c>
       <c r="D354" t="inlineStr"/>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
+          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
+          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
+          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
+          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
         </is>
       </c>
       <c r="D355" t="inlineStr"/>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
+          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
+          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
         </is>
       </c>
     </row>
@@ -12182,28 +12182,28 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
+          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
+          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
         </is>
       </c>
       <c r="D356" t="inlineStr"/>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
+          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
+          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
         </is>
       </c>
     </row>
@@ -12215,28 +12215,28 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
+          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
+          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
         </is>
       </c>
       <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
+          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
+          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
         </is>
       </c>
     </row>
@@ -12248,28 +12248,29 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
+          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
+          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
         </is>
       </c>
       <c r="D358" t="inlineStr"/>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
+          <t>nya tidak dilanjutkan," ucap Sudaryono.
+Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
+          <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
         </is>
       </c>
     </row>
@@ -12281,28 +12282,28 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
+          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
+          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
         </is>
       </c>
       <c r="D359" t="inlineStr"/>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
+          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
+          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
         </is>
       </c>
     </row>
@@ -12314,28 +12315,28 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
+          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
+          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
         </is>
       </c>
       <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
+          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
         </is>
       </c>
     </row>
@@ -12347,62 +12348,61 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
+          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
+          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
         </is>
       </c>
       <c r="D361" t="inlineStr"/>
       <c r="E361" t="inlineStr">
         <is>
-          <t>nya tidak dilanjutkan," ucap Sudaryono.
-Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
+          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>photo, top-news</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
+          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
         </is>
       </c>
       <c r="D362" t="inlineStr"/>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
+          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
+          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
         </is>
       </c>
     </row>
@@ -12414,28 +12414,28 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
+          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
         </is>
       </c>
       <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
+          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
+          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
         </is>
       </c>
     </row>
@@ -12447,61 +12447,61 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
+          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
+          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
         </is>
       </c>
       <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
+          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>photo, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
+          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
+          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
         </is>
       </c>
       <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
+          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12513,28 +12513,28 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
+          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
+          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
         </is>
       </c>
       <c r="D366" t="inlineStr"/>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
+          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
+          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12546,28 +12546,28 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
+          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
+          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
         </is>
       </c>
       <c r="D367" t="inlineStr"/>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
+          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
+          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
         </is>
       </c>
     </row>
@@ -12579,28 +12579,28 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
+          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
+          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
         </is>
       </c>
       <c r="D368" t="inlineStr"/>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
+          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
+          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
         </is>
       </c>
     </row>
@@ -12612,28 +12612,28 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
+          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
+          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
         </is>
       </c>
       <c r="D369" t="inlineStr"/>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
+          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
+          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12645,28 +12645,28 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
+          <t>Aktor senior Diding Boneng meninggal dunia</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
+          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
         </is>
       </c>
       <c r="D370" t="inlineStr"/>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
+          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12678,28 +12678,28 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
+          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
+          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
         </is>
       </c>
       <c r="D371" t="inlineStr"/>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12711,28 +12711,28 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
+          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
+          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
         </is>
       </c>
       <c r="D372" t="inlineStr"/>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
+          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
+          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12744,28 +12744,28 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Aktor senior Diding Boneng meninggal dunia</t>
+          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
+          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
         </is>
       </c>
       <c r="D373" t="inlineStr"/>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
+          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
         </is>
       </c>
     </row>
@@ -12777,28 +12777,28 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
+          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
+          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
         </is>
       </c>
       <c r="D374" t="inlineStr"/>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
+          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
+          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12810,28 +12810,28 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
+          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
+          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
         </is>
       </c>
       <c r="D375" t="inlineStr"/>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
+          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
         </is>
       </c>
     </row>
@@ -12843,28 +12843,28 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
+          <t>Harga bensin turun pada pekan pertama Agustus</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
+          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
         </is>
       </c>
       <c r="D376" t="inlineStr"/>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
+          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
+          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
         </is>
       </c>
     </row>
@@ -12876,127 +12876,127 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
+          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
+          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
         </is>
       </c>
       <c r="D377" t="inlineStr"/>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
+          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
+          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
+          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
+          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
         </is>
       </c>
       <c r="D378" t="inlineStr"/>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
+          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
+          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Harga bensin turun pada pekan pertama Agustus</t>
+          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
+          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
         </is>
       </c>
       <c r="D379" t="inlineStr"/>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
+          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
+          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
+          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
+          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
         </is>
       </c>
       <c r="D380" t="inlineStr"/>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
+          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
+          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
         </is>
       </c>
     </row>
@@ -13008,28 +13008,28 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
+          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
+          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
         </is>
       </c>
       <c r="D381" t="inlineStr"/>
       <c r="E381" t="inlineStr">
         <is>
-          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
+          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
         </is>
       </c>
     </row>
@@ -13041,28 +13041,28 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
+          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
+          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
         </is>
       </c>
       <c r="D382" t="inlineStr"/>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
+          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
+          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
         </is>
       </c>
     </row>
@@ -13074,28 +13074,28 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
+          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
+          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
         </is>
       </c>
       <c r="D383" t="inlineStr"/>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
+          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
         </is>
       </c>
     </row>
@@ -13107,28 +13107,28 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
+          <t>Menjaga pintu air perekonomian Indonesia</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
+          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
         </is>
       </c>
       <c r="D384" t="inlineStr"/>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
+          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
+          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
         </is>
       </c>
     </row>
@@ -13140,28 +13140,28 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
+          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
+          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
         </is>
       </c>
       <c r="D385" t="inlineStr"/>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
+          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
+          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
         </is>
       </c>
     </row>
@@ -13173,28 +13173,28 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
+          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
+          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
         </is>
       </c>
       <c r="D386" t="inlineStr"/>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
+          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
+          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
         </is>
       </c>
     </row>
@@ -13206,28 +13206,28 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Menjaga pintu air perekonomian Indonesia</t>
+          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
+          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
         </is>
       </c>
       <c r="D387" t="inlineStr"/>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
+          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
+          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
         </is>
       </c>
     </row>
@@ -13239,127 +13239,127 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
+          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
+          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
         </is>
       </c>
       <c r="D388" t="inlineStr"/>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
+          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
+          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
+          <t>Menteri PKP tegaskan KUR Perumahan perkuat ekonomi keluarga</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
+          <t>Mon, 03 Aug 2026 22:47:11 +0700</t>
         </is>
       </c>
       <c r="D389" t="inlineStr"/>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
+          <t>Menteri Perumahan dan Kawasan Permukiman (PKP) Maruarar Sirait menegaskan bahwa Kredit Usaha Rakyat (KUR) Perumahan ...</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5678465/menteri-pkp-tegaskan-kur-perumahan-perkuat-ekonomi-keluarga</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1321013.jpg</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
+          <t>Ekonom: Inflasi mereda, semester II jadi momentum jaga keseimbangan</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
+          <t>Mon, 03 Aug 2026 22:34:25 +0700</t>
         </is>
       </c>
       <c r="D390" t="inlineStr"/>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
+          <t>Kepala Ekonom Trimegah Sekuritas Indonesia Fakhrul Fulvian menilai semester II-2026 menjadi momentum untuk menjaga ...</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
+          <t>https://www.antaranews.com/berita/5678439/ekonom-inflasi-mereda-semester-ii-jadi-momentum-jaga-keseimbangan</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/21/IMG_2637.jpeg</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
+          <t>Pemkab Aceh Tenggara batasi pembelian BBM untuk cegah penimbunan</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
+          <t>Mon, 03 Aug 2026 22:25:13 +0700</t>
         </is>
       </c>
       <c r="D391" t="inlineStr"/>
       <c r="E391" t="inlineStr">
         <is>
-          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
+          <t>Pemerintah Kabupaten Aceh Tenggara bersama Forkopimda setempat saat ini telah melakukan pembatasan pembelian bahan ...</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5678431/pemkab-aceh-tenggara-batasi-pembelian-bbm-untuk-cegah-penimbunan</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-Bupati-Aceh-Tenggara-HM-Salim-Fakhry.jpeg</t>
         </is>
       </c>
     </row>
@@ -13371,28 +13371,28 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Gubernur tegaskan Sumut siap jadi pusat fashion Indonesia lewat wastra</t>
+          <t>MTI dorong kemudahan transaksi nirsentuh di MRT Jakarta</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:37:04 +0700</t>
+          <t>Mon, 03 Aug 2026 22:24:07 +0700</t>
         </is>
       </c>
       <c r="D392" t="inlineStr"/>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution menegaskan kesiapan Provinsi Sumut menjadi salah satu pusat fashion ...</t>
+          <t>PT Mitra Transaksi Indonesia (MTI) atau YOKKE mendukung penerapan sistem pembayaran kartu nirsentuh berbasis Europay, ...</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678355/gubernur-tegaskan-sumut-siap-jadi-pusat-fashion-indonesia-lewat-wastra</t>
+          <t>https://www.antaranews.com/berita/5678427/mti-dorong-kemudahan-transaksi-nirsentuh-di-mrt-jakarta</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001029105.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.59.08.jpeg</t>
         </is>
       </c>
     </row>
@@ -13404,28 +13404,28 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Kapal BBM bermuatan 7.600 kiloliter masuk Lombok</t>
+          <t>Gubernur tegaskan Sumut siap jadi pusat fashion Indonesia lewat wastra</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:32:28 +0700</t>
+          <t>Mon, 03 Aug 2026 21:37:04 +0700</t>
         </is>
       </c>
       <c r="D393" t="inlineStr"/>
       <c r="E393" t="inlineStr">
         <is>
-          <t>PT Pertamina Patra Niaga mendatangkan kapal pengangkut bahan bakar minyak (BBM) dengan total muatan 7.600 kiloliter ...</t>
+          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution menegaskan kesiapan Provinsi Sumut menjadi salah satu pusat fashion ...</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678341/kapal-bbm-bermuatan-7600-kiloliter-masuk-lombok</t>
+          <t>https://www.antaranews.com/berita/5678355/gubernur-tegaskan-sumut-siap-jadi-pusat-fashion-indonesia-lewat-wastra</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001432720.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001029105.jpg</t>
         </is>
       </c>
     </row>
@@ -13437,28 +13437,28 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Whoosh-kereta api dominasi jalur masuk wisatawan mancanegara di Jabar</t>
+          <t>Kapal BBM bermuatan 7.600 kiloliter masuk Lombok</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:28:59 +0700</t>
+          <t>Mon, 03 Aug 2026 21:32:28 +0700</t>
         </is>
       </c>
       <c r="D394" t="inlineStr"/>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Integrasi transportasi berbasis rel seperti Kereta Cepat Whoosh dan kereta api (KA) konvensional kian mengukuhkan ...</t>
+          <t>PT Pertamina Patra Niaga mendatangkan kapal pengangkut bahan bakar minyak (BBM) dengan total muatan 7.600 kiloliter ...</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678332/whoosh-kereta-api-dominasi-jalur-masuk-wisatawan-mancanegara-di-jabar</t>
+          <t>https://www.antaranews.com/berita/5678341/kapal-bbm-bermuatan-7600-kiloliter-masuk-lombok</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1002076644.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001432720.jpg</t>
         </is>
       </c>
     </row>
@@ -13470,61 +13470,61 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Daop 6 Yogyakarta tutup perlintasan tak terjaga Petak Sentolo–Rewulu</t>
+          <t>Whoosh-kereta api dominasi jalur masuk wisatawan mancanegara di Jabar</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:28:06 +0700</t>
+          <t>Mon, 03 Aug 2026 21:28:59 +0700</t>
         </is>
       </c>
       <c r="D395" t="inlineStr"/>
       <c r="E395" t="inlineStr">
         <is>
-          <t>PT Kereta Api Indonesia (Persero) Daerah Operasi 6 Yogyakarta terus berkolaborasi dengan pemerintah terkait, untuk ...</t>
+          <t>Integrasi transportasi berbasis rel seperti Kereta Cepat Whoosh dan kereta api (KA) konvensional kian mengukuhkan ...</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678331/daop-6-yogyakarta-tutup-perlintasan-tak-terjaga-petak-sentolo-rewulu</t>
+          <t>https://www.antaranews.com/berita/5678332/whoosh-kereta-api-dominasi-jalur-masuk-wisatawan-mancanegara-di-jabar</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029465.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1002076644.jpg</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis</t>
+          <t>ekonomi-bursa</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Kementan usulkan telur masuk skema CPP demi lindungi peternak rakyat</t>
+          <t>BEI terbitkan aturan emiten belum penuhi "free float" dapat notasi "P"</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:27:37 +0700</t>
+          <t>Mon, 03 Aug 2026 22:18:19 +0700</t>
         </is>
       </c>
       <c r="D396" t="inlineStr"/>
       <c r="E396" t="inlineStr">
         <is>
-          <t>Kementerian Pertanian (Kementan) mengusulkan komoditas telur ayam masuk dalam skema pengadaan Cadangan Pangan ...</t>
+          <t>PT Bursa Efek Indonesia (BEI) efektif memberlakukan dua Surat Edaran (SE) perihal Penambahan Tampilan Informasi Notasi ...</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678329/kementan-usulkan-telur-masuk-skema-cpp-demi-lindungi-peternak-rakyat</t>
+          <t>https://www.antaranews.com/berita/5678425/bei-terbitkan-aturan-emiten-belum-penuhi-free-float-dapat-notasi-p</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/9C2BC3E9-1C7E-4159-8805-C378B9294E25.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-01.jpg</t>
         </is>
       </c>
     </row>
@@ -13536,28 +13536,28 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>BEI terbitkan aturan emiten belum penuhi "free float" dapat notasi "P"</t>
+          <t>OJK bertemu 100 investor global, apresiasi reformasi pasar modal RI</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:18:19 +0700</t>
+          <t>Mon, 03 Aug 2026 21:29:14 +0700</t>
         </is>
       </c>
       <c r="D397" t="inlineStr"/>
       <c r="E397" t="inlineStr">
         <is>
-          <t>PT Bursa Efek Indonesia (BEI) efektif memberlakukan dua Surat Edaran (SE) perihal Penambahan Tampilan Informasi Notasi ...</t>
+          <t>Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Friderica Widyasari Dewi mengungkapkan bahwa OJK baru saja ...</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678425/bei-terbitkan-aturan-emiten-belum-penuhi-free-float-dapat-notasi-p</t>
+          <t>https://www.antaranews.com/berita/5678337/ojk-bertemu-100-investor-global-apresiasi-reformasi-pasar-modal-ri</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-270726-dr-01.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_2.jpeg</t>
         </is>
       </c>
     </row>
@@ -13569,28 +13569,28 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>OJK bertemu 100 investor global, apresiasi reformasi pasar modal RI</t>
+          <t>OJK: Pasar modal jaga peran sumber pembiayaan di tengah gejolak global</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:29:14 +0700</t>
+          <t>Mon, 03 Aug 2026 18:33:35 +0700</t>
         </is>
       </c>
       <c r="D398" t="inlineStr"/>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Friderica Widyasari Dewi mengungkapkan bahwa OJK baru saja ...</t>
+          <t>Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Friderica Widyasari Dewi alias Kiki memastikan bahwa pasar modal ...</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678337/ojk-bertemu-100-investor-global-apresiasi-reformasi-pasar-modal-ri</t>
+          <t>https://www.antaranews.com/berita/5677944/ojk-pasar-modal-jaga-peran-sumber-pembiayaan-di-tengah-gejolak-global</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_2.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18.jpeg</t>
         </is>
       </c>
     </row>
@@ -13602,28 +13602,28 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>OJK: Pasar modal jaga peran sumber pembiayaan di tengah gejolak global</t>
+          <t>IHSG awal pekan berpotensi variatif seiring sentimen global-domestik</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:33:35 +0700</t>
+          <t>Mon, 03 Aug 2026 09:42:28 +0700</t>
         </is>
       </c>
       <c r="D399" t="inlineStr"/>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Friderica Widyasari Dewi alias Kiki memastikan bahwa pasar modal ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Senin berpotensi bergerak variatif dipicu oleh ...</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677944/ojk-pasar-modal-jaga-peran-sumber-pembiayaan-di-tengah-gejolak-global</t>
+          <t>https://www.antaranews.com/berita/5677104/ihsg-awal-pekan-berpotensi-variatif-seiring-sentimen-global-domestik</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/12/ihsg-ditutup-menguat-2688871.jpg</t>
         </is>
       </c>
     </row>
@@ -13635,94 +13635,94 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>IHSG awal pekan berpotensi variatif seiring sentimen global-domestik</t>
+          <t>IHSG Senin dibuka menguat 36,49 poin ke posisi 6.272</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:42:28 +0700</t>
+          <t>Mon, 03 Aug 2026 09:11:26 +0700</t>
         </is>
       </c>
       <c r="D400" t="inlineStr"/>
       <c r="E400" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Senin berpotensi bergerak variatif dipicu oleh ...</t>
+          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Senin pagi dibuka menguat 36,49 poin atau 0,59 ...</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677104/ihsg-awal-pekan-berpotensi-variatif-seiring-sentimen-global-domestik</t>
+          <t>https://www.antaranews.com/berita/5677071/ihsg-senin-dibuka-menguat-3649-poin-ke-posisi-6272</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/12/12/ihsg-ditutup-menguat-2688871.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-2828631.jpg</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>ekonomi-bursa</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>IHSG Senin dibuka menguat 36,49 poin ke posisi 6.272</t>
+          <t>Bantuan beras 30 kg cair mulai 17 Agustus 2026, ini jadwal dan cara cek penerimanya</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:11:26 +0700</t>
+          <t>Mon, 03 Aug 2026 13:27:14 +0700</t>
         </is>
       </c>
       <c r="D401" t="inlineStr"/>
       <c r="E401" t="inlineStr">
         <is>
-          <t>Indeks Harga Saham Gabungan (IHSG) Bursa Efek Indonesia (BEI) pada Senin pagi dibuka menguat 36,49 poin atau 0,59 ...</t>
+          <t>Pemerintah memastikan penyaluran bantuan pangan beras tahap II tahun 2026 akan dimulai pada 17 Agustus 2026. Bantuan ...</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677071/ihsg-senin-dibuka-menguat-3649-poin-ke-posisi-6272</t>
+          <t>https://www.antaranews.com/berita/5677341/bantuan-beras-30-kg-cair-mulai-17-agustus-2026-ini-jadwal-dan-cara-cek-penerimanya</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/pergerakan-indeks-harga-saham-gabungan-2828631.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/26/kemensos-percepat-penyaluran-bansos-pkh-dan-bpnt-2778877.jpg</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>lifestyle</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Bantuan beras 30 kg cair mulai 17 Agustus 2026, ini jadwal dan cara cek penerimanya</t>
+          <t>10 ide usaha menjelang 17 Agustus 2026 yang berpotensi laris dan menguntungkan</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:27:14 +0700</t>
+          <t>Mon, 03 Aug 2026 18:16:58 +0700</t>
         </is>
       </c>
       <c r="D402" t="inlineStr"/>
       <c r="E402" t="inlineStr">
         <is>
-          <t>Pemerintah memastikan penyaluran bantuan pangan beras tahap II tahun 2026 akan dimulai pada 17 Agustus 2026. Bantuan ...</t>
+          <t>Momentum peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 dapat menjadi peluang bagi pelaku ...</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677341/bantuan-beras-30-kg-cair-mulai-17-agustus-2026-ini-jadwal-dan-cara-cek-penerimanya</t>
+          <t>https://www.antaranews.com/berita/5677896/10-ide-usaha-menjelang-17-agustus-2026-yang-berpotensi-laris-dan-menguntungkan</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/26/kemensos-percepat-penyaluran-bansos-pkh-dan-bpnt-2778877.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/08/02/sentra-penjualan-bendera-merah-putih-di-surabaya-020824-Ds-3.jpg</t>
         </is>
       </c>
     </row>
@@ -13734,28 +13734,28 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>10 ide usaha menjelang 17 Agustus 2026 yang berpotensi laris dan menguntungkan</t>
+          <t>10 ide lomba 17 Agustus untuk anak PAUD dan TK yang seru, edukatif, dan mudah digelar</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:16:58 +0700</t>
+          <t>Mon, 03 Aug 2026 13:38:29 +0700</t>
         </is>
       </c>
       <c r="D403" t="inlineStr"/>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Momentum peringatan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 dapat menjadi peluang bagi pelaku ...</t>
+          <t>Perayaan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 dapat menjadi momen bagi anak usia PAUD dan TK ...</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677896/10-ide-usaha-menjelang-17-agustus-2026-yang-berpotensi-laris-dan-menguntungkan</t>
+          <t>https://www.antaranews.com/berita/5677368/10-ide-lomba-17-agustus-untuk-anak-paud-dan-tk-yang-seru-edukatif-dan-mudah-digelar</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/08/02/sentra-penjualan-bendera-merah-putih-di-surabaya-020824-Ds-3.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/08/03/WhatsApp-Image-2024-08-03-at-20.37.28.jpeg</t>
         </is>
       </c>
     </row>
@@ -13767,28 +13767,28 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>10 ide lomba 17 Agustus untuk anak PAUD dan TK yang seru, edukatif, dan mudah digelar</t>
+          <t>Sering terbangun tengah malam? Kenali 7 penyebab dan cara mengatasinya</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:38:29 +0700</t>
+          <t>Mon, 03 Aug 2026 13:35:20 +0700</t>
         </is>
       </c>
       <c r="D404" t="inlineStr"/>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Perayaan HUT ke-81 Kemerdekaan Republik Indonesia pada 17 Agustus 2026 dapat menjadi momen bagi anak usia PAUD dan TK ...</t>
+          <t>Bangun di tengah malam sesekali merupakan hal yang normal. Namun, jika kondisi ini terjadi hampir setiap malam dan ...</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677368/10-ide-lomba-17-agustus-untuk-anak-paud-dan-tk-yang-seru-edukatif-dan-mudah-digelar</t>
+          <t>https://www.antaranews.com/berita/5677357/sering-terbangun-tengah-malam-kenali-7-penyebab-dan-cara-mengatasinya</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/08/03/WhatsApp-Image-2024-08-03-at-20.37.28.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/20/Penumpang-rela-menginap-menunggu-kereta-pertama-di-Stasiun-Cikarang-150726-ryl-5.jpg</t>
         </is>
       </c>
     </row>
@@ -13800,28 +13800,28 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>Sering terbangun tengah malam? Kenali 7 penyebab dan cara mengatasinya</t>
+          <t>Bahaya paparan pornografi pada anak: Dampak bagi otak, mental, dan perilaku</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:35:20 +0700</t>
+          <t>Mon, 03 Aug 2026 13:23:03 +0700</t>
         </is>
       </c>
       <c r="D405" t="inlineStr"/>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Bangun di tengah malam sesekali merupakan hal yang normal. Namun, jika kondisi ini terjadi hampir setiap malam dan ...</t>
+          <t>Perkembangan teknologi membuat anak-anak dan remaja semakin akrab dengan internet sejak usia dini. Di satu sisi, ...</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677357/sering-terbangun-tengah-malam-kenali-7-penyebab-dan-cara-mengatasinya</t>
+          <t>https://www.antaranews.com/berita/5677332/bahaya-paparan-pornografi-pada-anak-dampak-bagi-otak-mental-dan-perilaku</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/20/Penumpang-rela-menginap-menunggu-kereta-pertama-di-Stasiun-Cikarang-150726-ryl-5.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/02/ilustrasi-konten-berbau-pornografi.jpg</t>
         </is>
       </c>
     </row>
@@ -13833,28 +13833,28 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>Bahaya paparan pornografi pada anak: Dampak bagi otak, mental, dan perilaku</t>
+          <t>Sudah ngantuk tapi sulit tidur pulas? Ini penyebab dan cara atasinya</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:23:03 +0700</t>
+          <t>Mon, 03 Aug 2026 11:28:54 +0700</t>
         </is>
       </c>
       <c r="D406" t="inlineStr"/>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Perkembangan teknologi membuat anak-anak dan remaja semakin akrab dengan internet sejak usia dini. Di satu sisi, ...</t>
+          <t>Rasa kantuk yang muncul di malam hari seharusnya menjadi pertanda bahwa tubuh siap beristirahat. Namun, tidak sedikit ...</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677332/bahaya-paparan-pornografi-pada-anak-dampak-bagi-otak-mental-dan-perilaku</t>
+          <t>https://www.antaranews.com/berita/5677203/sudah-ngantuk-tapi-sulit-tidur-pulas-ini-penyebab-dan-cara-atasinya</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/02/ilustrasi-konten-berbau-pornografi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/17/Nafas.jpeg</t>
         </is>
       </c>
     </row>
@@ -13866,94 +13866,94 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>Sudah ngantuk tapi sulit tidur pulas? Ini penyebab dan cara atasinya</t>
+          <t>Cara cepat tidur dalam 5 menit, efektif untuk yang sulit pulas</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:28:54 +0700</t>
+          <t>Mon, 03 Aug 2026 11:25:40 +0700</t>
         </is>
       </c>
       <c r="D407" t="inlineStr"/>
       <c r="E407" t="inlineStr">
         <is>
-          <t>Rasa kantuk yang muncul di malam hari seharusnya menjadi pertanda bahwa tubuh siap beristirahat. Namun, tidak sedikit ...</t>
+          <t>Sulit tidur meski badan sudah terasa lelah merupakan masalah yang kerap dialami banyak orang. Kondisi ini sering ...</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677203/sudah-ngantuk-tapi-sulit-tidur-pulas-ini-penyebab-dan-cara-atasinya</t>
+          <t>https://www.antaranews.com/berita/5677199/cara-cepat-tidur-dalam-5-menit-efektif-untuk-yang-sulit-pulas</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/17/Nafas.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/04/tidua.jpg</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>lifestyle</t>
+          <t>tekno</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Cara cepat tidur dalam 5 menit, efektif untuk yang sulit pulas</t>
+          <t>Cara mengganti password WiFi lewat HP dan laptop dengan mudah</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:25:40 +0700</t>
+          <t>Mon, 03 Aug 2026 13:16:14 +0700</t>
         </is>
       </c>
       <c r="D408" t="inlineStr"/>
       <c r="E408" t="inlineStr">
         <is>
-          <t>Sulit tidur meski badan sudah terasa lelah merupakan masalah yang kerap dialami banyak orang. Kondisi ini sering ...</t>
+          <t>WiFi yang tiba-tiba terasa lambat padahal sinyal penuh dan kuota internet masih banyak tentu membuat kesal. Salah satu ...</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677199/cara-cepat-tidur-dalam-5-menit-efektif-untuk-yang-sulit-pulas</t>
+          <t>https://www.antaranews.com/berita/5677312/cara-mengganti-password-wifi-lewat-hp-dan-laptop-dengan-mudah</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/11/04/tidua.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/08/19/antarafoto-warga-sediakan-internet-gratis-bagi-pelajar-190820-ief-2-1.jpg</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>tekno</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Cara mengganti password WiFi lewat HP dan laptop dengan mudah</t>
+          <t>Piala AFF 2026 : Indonesia takluk 0-3 dari Vietnam</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:16:14 +0700</t>
+          <t>Mon, 03 Aug 2026 22:26:45 +0700</t>
         </is>
       </c>
       <c r="D409" t="inlineStr"/>
       <c r="E409" t="inlineStr">
         <is>
-          <t>WiFi yang tiba-tiba terasa lambat padahal sinyal penuh dan kuota internet masih banyak tentu membuat kesal. Salah satu ...</t>
+          <t>Pelatih Timnas Indonesia Jhon Herdman memberikan arahan kepada anak didiknya saat melawan Timnas Vietnam pada pertandingan Grup A Piala AFF 2026 di Stadion Pakansari, Kabupaten Bogor, Jawa Barat, Senin (3/8/2026). ANTARA FOTO/Bayu Pratama S/mrh/wsj.</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677312/cara-mengganti-password-wifi-lewat-hp-dan-laptop-dengan-mudah</t>
+          <t>https://www.antaranews.com/foto/5678435/piala-aff-2026-indonesia-takluk-0-3-dari-vietnam</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2020/08/19/antarafoto-warga-sediakan-internet-gratis-bagi-pelajar-190820-ief-2-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/255x170/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-11b.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-03 20:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-03.xlsx
+++ b/data/berita_antara_2026-08-03.xlsx
@@ -10961,28 +10961,28 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
+          <t>Prabowo-PM Thailand perkuat kemitraan strategis ASEAN</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
+          <t>Mon, 03 Aug 2026 22:52:55 +0700</t>
         </is>
       </c>
       <c r="D319" t="inlineStr"/>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
+          <t>Presiden RI Prabowo Subianto dan Perdana Menteri (PM) Thailand Anutin Charnvirakul sepakat memperkuat kemitraan ...</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
+          <t>https://www.antaranews.com/berita/5678476/prabowo-pm-thailand-perkuat-kemitraan-strategis-asean</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_F6F7E006D3CC-1.jpeg</t>
         </is>
       </c>
     </row>
@@ -10994,94 +10994,94 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
+          <t>Galaxy Tab S12 Ultra mejeng di Geekbench, hadir dengan Dimensity 9500</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
+          <t>Mon, 03 Aug 2026 22:48:03 +0700</t>
         </is>
       </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
+          <t>Samsung Galaxy Tab S12 Ultra dalam seri perangkat Galaxy Tab S12 yang diperkirakan dirilis September 2026 muncul di ...</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
+          <t>https://www.antaranews.com/berita/5678469/galaxy-tab-s12-ultra-mejeng-di-geekbench-hadir-dengan-dimensity-9500</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/InShot_20260803_215836626.jpg</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
+          <t>Whoosh-kereta api dominasi jalur masuk wisatawan mancanegara di Jabar</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
+          <t>Mon, 03 Aug 2026 21:28:59 +0700</t>
         </is>
       </c>
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr">
         <is>
-          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
+          <t>Integrasi transportasi berbasis rel seperti Kereta Cepat Whoosh dan kereta api (KA) konvensional kian mengukuhkan ...</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
+          <t>https://www.antaranews.com/berita/5678332/whoosh-kereta-api-dominasi-jalur-masuk-wisatawan-mancanegara-di-jabar</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1002076644.jpg</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
+          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
         </is>
       </c>
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
+          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
+          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
         </is>
       </c>
     </row>
@@ -11093,61 +11093,61 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
+          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
         </is>
       </c>
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
+          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
+          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
+          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
+          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
         </is>
       </c>
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
+          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
+          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
         </is>
       </c>
     </row>
@@ -11159,94 +11159,94 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
+          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
+          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
         </is>
       </c>
       <c r="D325" t="inlineStr"/>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
+          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
+          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
+          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
+          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
         </is>
       </c>
       <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr">
         <is>
-          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
+          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
+          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
+          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
+          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
         </is>
       </c>
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
+          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
+          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
         </is>
       </c>
     </row>
@@ -11258,61 +11258,61 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
+          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
+          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
         </is>
       </c>
       <c r="D328" t="inlineStr"/>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
+          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
+          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
+          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
+          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
         </is>
       </c>
       <c r="D329" t="inlineStr"/>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
+          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
+          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
         </is>
       </c>
     </row>
@@ -11324,28 +11324,28 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
+          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
+          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
         </is>
       </c>
       <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr">
         <is>
-          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
+          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
+          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11357,28 +11357,28 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
+          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr">
         <is>
-          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
+          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
+          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11390,28 +11390,28 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
+          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
+          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
+          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
         </is>
       </c>
     </row>
@@ -11423,28 +11423,28 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
+          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
+          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
+          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
         </is>
       </c>
     </row>
@@ -11456,61 +11456,61 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
+          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
         </is>
       </c>
       <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
+          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
+          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
+          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
         </is>
       </c>
       <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
+          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
+          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11522,94 +11522,94 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
+          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
+          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
+          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
+          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
+          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
+          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
+          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
+          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
         </is>
       </c>
       <c r="D338" t="inlineStr"/>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
+          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
+          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
         </is>
       </c>
     </row>
@@ -11621,61 +11621,61 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
+          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
+          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
+          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
+          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
+          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
+          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
         </is>
       </c>
     </row>
@@ -11687,28 +11687,28 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
+          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
+          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
+          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
+          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
         </is>
       </c>
     </row>
@@ -11720,94 +11720,94 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Presiden Prabowo terima kunjungan PM Thailand di Istana Merdeka</t>
+          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:59:27 +0700</t>
+          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr">
         <is>
-          <t>ANTARA - Presiden Prabowo Subianto menerima kunjungan resmi Perdana Menteri Thailand Anutin Charnvirakul di Istana ...</t>
+          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678461/presiden-prabowo-terima-kunjungan-pm-thailand-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRESIDEN-PRABOWO-TERIMA-KUNJUNGAN-PM-THAILAND-DI-ISTANA-MERDEKA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Basarnas jemput 66 korban KM Mutiara Sentosa II dari Masalembu</t>
+          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:58:38 +0700</t>
+          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
       <c r="E343" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) mengerahkan satu unit kapal untuk menjemput 66 korban ...</t>
+          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678472/basarnas-jemput-66-korban-km-mutiara-sentosa-ii-dari-masalembu</t>
+          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BASARNAS-JEMPUT-66-KORBAN-KM-MUTIARA-SENTOSA-II-DARI-MASALEMBU.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Kementerian ATR/BPN telah terbitkan 124 ribu SK sertifikat rumah MBR</t>
+          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:56:36 +0700</t>
+          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) menyatakan telah menerbitkan surat keputusan ...</t>
+          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678484/kementerian-atr-bpn-telah-terbitkan-124-ribu-sk-sertifikat-rumah-mbr</t>
+          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_224532.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
         </is>
       </c>
     </row>
@@ -11819,28 +11819,28 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Timnas Indonesia dibungkam Vietnam 0-3</t>
+          <t>Presiden Prabowo terima kunjungan PM Thailand di Istana Merdeka</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:54:01 +0700</t>
+          <t>Mon, 03 Aug 2026 22:59:27 +0700</t>
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Timnas Indonesia dibungkam Vietnam 0-3 di kandang pada laga lanjutan Grup A Piala AFF 2026 di Stadion Pakansari, Bogor, ...</t>
+          <t>ANTARA - Presiden Prabowo Subianto menerima kunjungan resmi Perdana Menteri Thailand Anutin Charnvirakul di Istana ...</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678480/timnas-indonesia-dibungkam-vietnam-0-3</t>
+          <t>https://www.antaranews.com/video/5678461/presiden-prabowo-terima-kunjungan-pm-thailand-di-istana-merdeka</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-21a.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRESIDEN-PRABOWO-TERIMA-KUNJUNGAN-PM-THAILAND-DI-ISTANA-MERDEKA.jpg</t>
         </is>
       </c>
     </row>
@@ -11852,94 +11852,94 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Prabowo-PM Thailand perkuat kemitraan strategis ASEAN</t>
+          <t>Basarnas jemput 66 korban KM Mutiara Sentosa II dari Masalembu</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:52:55 +0700</t>
+          <t>Mon, 03 Aug 2026 22:58:38 +0700</t>
         </is>
       </c>
       <c r="D346" t="inlineStr"/>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Presiden RI Prabowo Subianto dan Perdana Menteri (PM) Thailand Anutin Charnvirakul sepakat memperkuat kemitraan ...</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) mengerahkan satu unit kapal untuk menjemput 66 korban ...</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678476/prabowo-pm-thailand-perkuat-kemitraan-strategis-asean</t>
+          <t>https://www.antaranews.com/video/5678472/basarnas-jemput-66-korban-km-mutiara-sentosa-ii-dari-masalembu</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_F6F7E006D3CC-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BASARNAS-JEMPUT-66-KORBAN-KM-MUTIARA-SENTOSA-II-DARI-MASALEMBU.jpg</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Galaxy Tab S12 Ultra mejeng di Geekbench, hadir dengan Dimensity 9500</t>
+          <t>Kementerian ATR/BPN telah terbitkan 124 ribu SK sertifikat rumah MBR</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:48:03 +0700</t>
+          <t>Mon, 03 Aug 2026 22:56:36 +0700</t>
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Samsung Galaxy Tab S12 Ultra dalam seri perangkat Galaxy Tab S12 yang diperkirakan dirilis September 2026 muncul di ...</t>
+          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) menyatakan telah menerbitkan surat keputusan ...</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678469/galaxy-tab-s12-ultra-mejeng-di-geekbench-hadir-dengan-dimensity-9500</t>
+          <t>https://www.antaranews.com/berita/5678484/kementerian-atr-bpn-telah-terbitkan-124-ribu-sk-sertifikat-rumah-mbr</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/InShot_20260803_215836626.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_224532.jpg</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
+          <t>Timnas Indonesia dibungkam Vietnam 0-3</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
+          <t>Mon, 03 Aug 2026 22:54:01 +0700</t>
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
+          <t>Timnas Indonesia dibungkam Vietnam 0-3 di kandang pada laga lanjutan Grup A Piala AFF 2026 di Stadion Pakansari, Bogor, ...</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
+          <t>https://www.antaranews.com/berita/5678480/timnas-indonesia-dibungkam-vietnam-0-3</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-21a.jpg</t>
         </is>
       </c>
     </row>
@@ -11951,160 +11951,160 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
+          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
+          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
         </is>
       </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
+          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
+          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
+          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
+          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
         </is>
       </c>
       <c r="D350" t="inlineStr"/>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
+          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
+          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
+          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
+          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
         </is>
       </c>
       <c r="D351" t="inlineStr"/>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
+          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
+          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
+          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
         </is>
       </c>
       <c r="D352" t="inlineStr"/>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
+          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
+          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
+          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
+          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
+          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12116,28 +12116,28 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
+          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
+          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
         </is>
       </c>
       <c r="D354" t="inlineStr"/>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
+          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
         </is>
       </c>
     </row>
@@ -12149,28 +12149,28 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
+          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
+          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
         </is>
       </c>
       <c r="D355" t="inlineStr"/>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
+          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
+          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
         </is>
       </c>
     </row>
@@ -12182,28 +12182,28 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
+          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
+          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
         </is>
       </c>
       <c r="D356" t="inlineStr"/>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
+          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
+          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
         </is>
       </c>
     </row>
@@ -12215,28 +12215,28 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
+          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
+          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
         </is>
       </c>
       <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
+          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
         </is>
       </c>
     </row>
@@ -12248,62 +12248,62 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
+          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
+          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
         </is>
       </c>
       <c r="D358" t="inlineStr"/>
       <c r="E358" t="inlineStr">
         <is>
+          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>top-news</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr"/>
+      <c r="E359" t="inlineStr">
+        <is>
           <t>nya tidak dilanjutkan," ucap Sudaryono.
 Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
         </is>
       </c>
-      <c r="F358" t="inlineStr">
+      <c r="F359" t="inlineStr">
         <is>
           <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
         </is>
       </c>
-      <c r="G358" t="inlineStr">
+      <c r="G359" t="inlineStr">
         <is>
           <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" t="inlineStr">
-        <is>
-          <t>top-news</t>
-        </is>
-      </c>
-      <c r="B359" t="inlineStr">
-        <is>
-          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
-        </is>
-      </c>
-      <c r="C359" t="inlineStr">
-        <is>
-          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
-        </is>
-      </c>
-      <c r="D359" t="inlineStr"/>
-      <c r="E359" t="inlineStr">
-        <is>
-          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
-        </is>
-      </c>
-      <c r="F359" t="inlineStr">
-        <is>
-          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
-        </is>
-      </c>
-      <c r="G359" t="inlineStr">
-        <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
         </is>
       </c>
     </row>
@@ -12315,28 +12315,28 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
+          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
+          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
         </is>
       </c>
       <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
+          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
+          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
         </is>
       </c>
     </row>
@@ -12348,94 +12348,94 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
+          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
+          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
         </is>
       </c>
       <c r="D361" t="inlineStr"/>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
+          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
+          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>photo, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
+          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
+          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
         </is>
       </c>
       <c r="D362" t="inlineStr"/>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
+          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>photo, top-news</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
+          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
         </is>
       </c>
       <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
+          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
+          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
         </is>
       </c>
     </row>
@@ -12447,28 +12447,28 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
+          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
         </is>
       </c>
       <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
+          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
+          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
         </is>
       </c>
     </row>
@@ -12480,28 +12480,28 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
+          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
+          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
         </is>
       </c>
       <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
+          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
         </is>
       </c>
     </row>
@@ -12513,28 +12513,28 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
+          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
+          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
         </is>
       </c>
       <c r="D366" t="inlineStr"/>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
+          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12546,28 +12546,28 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
+          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
+          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
         </is>
       </c>
       <c r="D367" t="inlineStr"/>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
+          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12579,28 +12579,28 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
+          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
+          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
         </is>
       </c>
       <c r="D368" t="inlineStr"/>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
+          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
         </is>
       </c>
     </row>
@@ -12612,28 +12612,28 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
+          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
+          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
         </is>
       </c>
       <c r="D369" t="inlineStr"/>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
+          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
+          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
         </is>
       </c>
     </row>
@@ -12645,28 +12645,28 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Aktor senior Diding Boneng meninggal dunia</t>
+          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
+          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
         </is>
       </c>
       <c r="D370" t="inlineStr"/>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
+          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
+          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12678,28 +12678,28 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
+          <t>Aktor senior Diding Boneng meninggal dunia</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
+          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
         </is>
       </c>
       <c r="D371" t="inlineStr"/>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
+          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
+          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12711,28 +12711,28 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
+          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
+          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
         </is>
       </c>
       <c r="D372" t="inlineStr"/>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
+          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12744,28 +12744,28 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
+          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
+          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
         </is>
       </c>
       <c r="D373" t="inlineStr"/>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
+          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
+          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12777,28 +12777,28 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
+          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
+          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
         </is>
       </c>
       <c r="D374" t="inlineStr"/>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
+          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
         </is>
       </c>
     </row>
@@ -12810,28 +12810,28 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
+          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
+          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
         </is>
       </c>
       <c r="D375" t="inlineStr"/>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
+          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
+          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12843,28 +12843,28 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Harga bensin turun pada pekan pertama Agustus</t>
+          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
+          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
         </is>
       </c>
       <c r="D376" t="inlineStr"/>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
+          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
         </is>
       </c>
     </row>
@@ -12876,61 +12876,61 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
+          <t>Harga bensin turun pada pekan pertama Agustus</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
+          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
         </is>
       </c>
       <c r="D377" t="inlineStr"/>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
+          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
+          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
+          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
+          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
         </is>
       </c>
       <c r="D378" t="inlineStr"/>
       <c r="E378" t="inlineStr">
         <is>
-          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
+          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
+          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12942,28 +12942,28 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
+          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
+          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
         </is>
       </c>
       <c r="D379" t="inlineStr"/>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
+          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
+          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
         </is>
       </c>
     </row>
@@ -12975,28 +12975,28 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
+          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
+          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
         </is>
       </c>
       <c r="D380" t="inlineStr"/>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
+          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
+          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
         </is>
       </c>
     </row>
@@ -13008,28 +13008,28 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
+          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
+          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
         </is>
       </c>
       <c r="D381" t="inlineStr"/>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
+          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
+          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
         </is>
       </c>
     </row>
@@ -13041,28 +13041,28 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
+          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
+          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
         </is>
       </c>
       <c r="D382" t="inlineStr"/>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
+          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
         </is>
       </c>
     </row>
@@ -13074,28 +13074,28 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
+          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
+          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
         </is>
       </c>
       <c r="D383" t="inlineStr"/>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
+          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
+          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
         </is>
       </c>
     </row>
@@ -13107,28 +13107,28 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Menjaga pintu air perekonomian Indonesia</t>
+          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
+          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
         </is>
       </c>
       <c r="D384" t="inlineStr"/>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
         </is>
       </c>
     </row>
@@ -13140,28 +13140,28 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
+          <t>Menjaga pintu air perekonomian Indonesia</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
+          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
         </is>
       </c>
       <c r="D385" t="inlineStr"/>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
+          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
+          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
         </is>
       </c>
     </row>
@@ -13173,28 +13173,28 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
+          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
+          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
         </is>
       </c>
       <c r="D386" t="inlineStr"/>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
+          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
         </is>
       </c>
     </row>
@@ -13206,28 +13206,28 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
+          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
+          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
         </is>
       </c>
       <c r="D387" t="inlineStr"/>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
+          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
+          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
         </is>
       </c>
     </row>
@@ -13239,61 +13239,61 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
+          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
+          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
         </is>
       </c>
       <c r="D388" t="inlineStr"/>
       <c r="E388" t="inlineStr">
         <is>
-          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
+          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Menteri PKP tegaskan KUR Perumahan perkuat ekonomi keluarga</t>
+          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:47:11 +0700</t>
+          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
         </is>
       </c>
       <c r="D389" t="inlineStr"/>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Menteri Perumahan dan Kawasan Permukiman (PKP) Maruarar Sirait menegaskan bahwa Kredit Usaha Rakyat (KUR) Perumahan ...</t>
+          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678465/menteri-pkp-tegaskan-kur-perumahan-perkuat-ekonomi-keluarga</t>
+          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1321013.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
         </is>
       </c>
     </row>
@@ -13305,28 +13305,28 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Ekonom: Inflasi mereda, semester II jadi momentum jaga keseimbangan</t>
+          <t>Menteri PKP tegaskan KUR Perumahan perkuat ekonomi keluarga</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:34:25 +0700</t>
+          <t>Mon, 03 Aug 2026 22:47:11 +0700</t>
         </is>
       </c>
       <c r="D390" t="inlineStr"/>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Kepala Ekonom Trimegah Sekuritas Indonesia Fakhrul Fulvian menilai semester II-2026 menjadi momentum untuk menjaga ...</t>
+          <t>Menteri Perumahan dan Kawasan Permukiman (PKP) Maruarar Sirait menegaskan bahwa Kredit Usaha Rakyat (KUR) Perumahan ...</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678439/ekonom-inflasi-mereda-semester-ii-jadi-momentum-jaga-keseimbangan</t>
+          <t>https://www.antaranews.com/berita/5678465/menteri-pkp-tegaskan-kur-perumahan-perkuat-ekonomi-keluarga</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/01/21/IMG_2637.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1321013.jpg</t>
         </is>
       </c>
     </row>
@@ -13338,28 +13338,28 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Pemkab Aceh Tenggara batasi pembelian BBM untuk cegah penimbunan</t>
+          <t>Ekonom: Inflasi mereda, semester II jadi momentum jaga keseimbangan</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:25:13 +0700</t>
+          <t>Mon, 03 Aug 2026 22:34:25 +0700</t>
         </is>
       </c>
       <c r="D391" t="inlineStr"/>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Pemerintah Kabupaten Aceh Tenggara bersama Forkopimda setempat saat ini telah melakukan pembatasan pembelian bahan ...</t>
+          <t>Kepala Ekonom Trimegah Sekuritas Indonesia Fakhrul Fulvian menilai semester II-2026 menjadi momentum untuk menjaga ...</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678431/pemkab-aceh-tenggara-batasi-pembelian-bbm-untuk-cegah-penimbunan</t>
+          <t>https://www.antaranews.com/berita/5678439/ekonom-inflasi-mereda-semester-ii-jadi-momentum-jaga-keseimbangan</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-Bupati-Aceh-Tenggara-HM-Salim-Fakhry.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/01/21/IMG_2637.jpeg</t>
         </is>
       </c>
     </row>
@@ -13371,28 +13371,28 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>MTI dorong kemudahan transaksi nirsentuh di MRT Jakarta</t>
+          <t>Pemkab Aceh Tenggara batasi pembelian BBM untuk cegah penimbunan</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:24:07 +0700</t>
+          <t>Mon, 03 Aug 2026 22:25:13 +0700</t>
         </is>
       </c>
       <c r="D392" t="inlineStr"/>
       <c r="E392" t="inlineStr">
         <is>
-          <t>PT Mitra Transaksi Indonesia (MTI) atau YOKKE mendukung penerapan sistem pembayaran kartu nirsentuh berbasis Europay, ...</t>
+          <t>Pemerintah Kabupaten Aceh Tenggara bersama Forkopimda setempat saat ini telah melakukan pembatasan pembelian bahan ...</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678427/mti-dorong-kemudahan-transaksi-nirsentuh-di-mrt-jakarta</t>
+          <t>https://www.antaranews.com/berita/5678431/pemkab-aceh-tenggara-batasi-pembelian-bbm-untuk-cegah-penimbunan</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.59.08.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/20260803-Bupati-Aceh-Tenggara-HM-Salim-Fakhry.jpeg</t>
         </is>
       </c>
     </row>
@@ -13404,28 +13404,28 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Gubernur tegaskan Sumut siap jadi pusat fashion Indonesia lewat wastra</t>
+          <t>MTI dorong kemudahan transaksi nirsentuh di MRT Jakarta</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:37:04 +0700</t>
+          <t>Mon, 03 Aug 2026 22:24:07 +0700</t>
         </is>
       </c>
       <c r="D393" t="inlineStr"/>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution menegaskan kesiapan Provinsi Sumut menjadi salah satu pusat fashion ...</t>
+          <t>PT Mitra Transaksi Indonesia (MTI) atau YOKKE mendukung penerapan sistem pembayaran kartu nirsentuh berbasis Europay, ...</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678355/gubernur-tegaskan-sumut-siap-jadi-pusat-fashion-indonesia-lewat-wastra</t>
+          <t>https://www.antaranews.com/berita/5678427/mti-dorong-kemudahan-transaksi-nirsentuh-di-mrt-jakarta</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001029105.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.59.08.jpeg</t>
         </is>
       </c>
     </row>
@@ -13437,28 +13437,28 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Kapal BBM bermuatan 7.600 kiloliter masuk Lombok</t>
+          <t>Gubernur tegaskan Sumut siap jadi pusat fashion Indonesia lewat wastra</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:32:28 +0700</t>
+          <t>Mon, 03 Aug 2026 21:37:04 +0700</t>
         </is>
       </c>
       <c r="D394" t="inlineStr"/>
       <c r="E394" t="inlineStr">
         <is>
-          <t>PT Pertamina Patra Niaga mendatangkan kapal pengangkut bahan bakar minyak (BBM) dengan total muatan 7.600 kiloliter ...</t>
+          <t>Gubernur Sumatera Utara (Sumut) Bobby Nasution menegaskan kesiapan Provinsi Sumut menjadi salah satu pusat fashion ...</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678341/kapal-bbm-bermuatan-7600-kiloliter-masuk-lombok</t>
+          <t>https://www.antaranews.com/berita/5678355/gubernur-tegaskan-sumut-siap-jadi-pusat-fashion-indonesia-lewat-wastra</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001432720.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001029105.jpg</t>
         </is>
       </c>
     </row>
@@ -13470,28 +13470,28 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Whoosh-kereta api dominasi jalur masuk wisatawan mancanegara di Jabar</t>
+          <t>Kapal BBM bermuatan 7.600 kiloliter masuk Lombok</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:28:59 +0700</t>
+          <t>Mon, 03 Aug 2026 21:32:28 +0700</t>
         </is>
       </c>
       <c r="D395" t="inlineStr"/>
       <c r="E395" t="inlineStr">
         <is>
-          <t>Integrasi transportasi berbasis rel seperti Kereta Cepat Whoosh dan kereta api (KA) konvensional kian mengukuhkan ...</t>
+          <t>PT Pertamina Patra Niaga mendatangkan kapal pengangkut bahan bakar minyak (BBM) dengan total muatan 7.600 kiloliter ...</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678332/whoosh-kereta-api-dominasi-jalur-masuk-wisatawan-mancanegara-di-jabar</t>
+          <t>https://www.antaranews.com/berita/5678341/kapal-bbm-bermuatan-7600-kiloliter-masuk-lombok</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1002076644.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1001432720.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-03 21:56 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-03.xlsx
+++ b/data/berita_antara_2026-08-03.xlsx
@@ -11060,28 +11060,28 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
+          <t>Presiden Prabowo terima kunjungan PM Thailand di Istana Merdeka</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
+          <t>Mon, 03 Aug 2026 22:59:27 +0700</t>
         </is>
       </c>
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
+          <t>ANTARA - Presiden Prabowo Subianto menerima kunjungan resmi Perdana Menteri Thailand Anutin Charnvirakul di Istana ...</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
+          <t>https://www.antaranews.com/video/5678461/presiden-prabowo-terima-kunjungan-pm-thailand-di-istana-merdeka</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRESIDEN-PRABOWO-TERIMA-KUNJUNGAN-PM-THAILAND-DI-ISTANA-MERDEKA.jpg</t>
         </is>
       </c>
     </row>
@@ -11093,28 +11093,28 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
+          <t>Basarnas jemput 66 korban KM Mutiara Sentosa II dari Masalembu</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
+          <t>Mon, 03 Aug 2026 22:58:38 +0700</t>
         </is>
       </c>
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
+          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) mengerahkan satu unit kapal untuk menjemput 66 korban ...</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
+          <t>https://www.antaranews.com/video/5678472/basarnas-jemput-66-korban-km-mutiara-sentosa-ii-dari-masalembu</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BASARNAS-JEMPUT-66-KORBAN-KM-MUTIARA-SENTOSA-II-DARI-MASALEMBU.jpg</t>
         </is>
       </c>
     </row>
@@ -11126,61 +11126,61 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
+          <t>Timnas Indonesia dibungkam Vietnam 0-3</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
+          <t>Mon, 03 Aug 2026 22:54:01 +0700</t>
         </is>
       </c>
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr">
         <is>
-          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
+          <t>Timnas Indonesia dibungkam Vietnam 0-3 di kandang pada laga lanjutan Grup A Piala AFF 2026 di Stadion Pakansari, Bogor, ...</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
+          <t>https://www.antaranews.com/berita/5678480/timnas-indonesia-dibungkam-vietnam-0-3</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-21a.jpg</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
+          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
         </is>
       </c>
       <c r="D325" t="inlineStr"/>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
+          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
+          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
         </is>
       </c>
     </row>
@@ -11192,61 +11192,61 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
+          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
         </is>
       </c>
       <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
+          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
+          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
+          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
+          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
         </is>
       </c>
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
+          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
+          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
         </is>
       </c>
     </row>
@@ -11258,94 +11258,94 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
+          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
+          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
         </is>
       </c>
       <c r="D328" t="inlineStr"/>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
+          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
+          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
+          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
+          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
         </is>
       </c>
       <c r="D329" t="inlineStr"/>
       <c r="E329" t="inlineStr">
         <is>
-          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
+          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
+          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
+          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
+          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
         </is>
       </c>
       <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
+          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
+          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
         </is>
       </c>
     </row>
@@ -11357,61 +11357,61 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
+          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
+          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
+          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
+          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
+          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
+          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
+          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
+          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
         </is>
       </c>
     </row>
@@ -11423,28 +11423,28 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
+          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
+          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
-          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
+          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
+          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11456,28 +11456,28 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
+          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
         </is>
       </c>
       <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr">
         <is>
-          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
+          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
+          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11489,28 +11489,28 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
+          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
         </is>
       </c>
       <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
+          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
+          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
         </is>
       </c>
     </row>
@@ -11522,28 +11522,28 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
+          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
       <c r="E336" t="inlineStr">
         <is>
-          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
+          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
+          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
         </is>
       </c>
     </row>
@@ -11555,61 +11555,61 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
+          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
+          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
+          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
+          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
         </is>
       </c>
       <c r="D338" t="inlineStr"/>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
+          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
+          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
         </is>
       </c>
     </row>
@@ -11621,94 +11621,94 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
+          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
+          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
+          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
+          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
+          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
+          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
+          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
+          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
+          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
+          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
         </is>
       </c>
     </row>
@@ -11720,61 +11720,61 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
+          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
+          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
+          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
+          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
+          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
+          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
         </is>
       </c>
     </row>
@@ -11786,28 +11786,28 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
+          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
+          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
+          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
+          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
         </is>
       </c>
     </row>
@@ -11819,127 +11819,127 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Presiden Prabowo terima kunjungan PM Thailand di Istana Merdeka</t>
+          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:59:27 +0700</t>
+          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
       <c r="E345" t="inlineStr">
         <is>
-          <t>ANTARA - Presiden Prabowo Subianto menerima kunjungan resmi Perdana Menteri Thailand Anutin Charnvirakul di Istana ...</t>
+          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678461/presiden-prabowo-terima-kunjungan-pm-thailand-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/PRESIDEN-PRABOWO-TERIMA-KUNJUNGAN-PM-THAILAND-DI-ISTANA-MERDEKA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Basarnas jemput 66 korban KM Mutiara Sentosa II dari Masalembu</t>
+          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:58:38 +0700</t>
+          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
         </is>
       </c>
       <c r="D346" t="inlineStr"/>
       <c r="E346" t="inlineStr">
         <is>
-          <t>ANTARA - Badan Pencarian dan Pertolongan Nasional (Basarnas) mengerahkan satu unit kapal untuk menjemput 66 korban ...</t>
+          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678472/basarnas-jemput-66-korban-km-mutiara-sentosa-ii-dari-masalembu</t>
+          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_BASARNAS-JEMPUT-66-KORBAN-KM-MUTIARA-SENTOSA-II-DARI-MASALEMBU.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Kementerian ATR/BPN telah terbitkan 124 ribu SK sertifikat rumah MBR</t>
+          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:56:36 +0700</t>
+          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) menyatakan telah menerbitkan surat keputusan ...</t>
+          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678484/kementerian-atr-bpn-telah-terbitkan-124-ribu-sk-sertifikat-rumah-mbr</t>
+          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_224532.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Timnas Indonesia dibungkam Vietnam 0-3</t>
+          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 22:54:01 +0700</t>
+          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Timnas Indonesia dibungkam Vietnam 0-3 di kandang pada laga lanjutan Grup A Piala AFF 2026 di Stadion Pakansari, Bogor, ...</t>
+          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678480/timnas-indonesia-dibungkam-vietnam-0-3</t>
+          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Timnas-Indonesia-lawan-Vietnam-030826-Bay-21a.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
         </is>
       </c>
     </row>
@@ -11951,160 +11951,160 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
+          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
+          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
         </is>
       </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
+          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
+          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
+          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
+          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
         </is>
       </c>
       <c r="D350" t="inlineStr"/>
       <c r="E350" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
+          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
+          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
+          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
         </is>
       </c>
       <c r="D351" t="inlineStr"/>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
+          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
+          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
+          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
+          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
         </is>
       </c>
       <c r="D352" t="inlineStr"/>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
+          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
+          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
+          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
+          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
         </is>
       </c>
     </row>
@@ -12116,28 +12116,28 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
+          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
+          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
         </is>
       </c>
       <c r="D354" t="inlineStr"/>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
+          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
+          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
         </is>
       </c>
     </row>
@@ -12149,28 +12149,28 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
+          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
+          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
         </is>
       </c>
       <c r="D355" t="inlineStr"/>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
+          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
+          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
         </is>
       </c>
     </row>
@@ -12182,28 +12182,28 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
+          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
+          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
         </is>
       </c>
       <c r="D356" t="inlineStr"/>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
+          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
+          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
         </is>
       </c>
     </row>
@@ -12215,28 +12215,28 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
+          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
+          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
         </is>
       </c>
       <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
+          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
+          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
         </is>
       </c>
     </row>
@@ -12248,28 +12248,29 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
+          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
+          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
         </is>
       </c>
       <c r="D358" t="inlineStr"/>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
+          <t>nya tidak dilanjutkan," ucap Sudaryono.
+Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
         </is>
       </c>
     </row>
@@ -12281,29 +12282,28 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
+          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
+          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
         </is>
       </c>
       <c r="D359" t="inlineStr"/>
       <c r="E359" t="inlineStr">
         <is>
-          <t>nya tidak dilanjutkan," ucap Sudaryono.
-Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
+          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
+          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
         </is>
       </c>
     </row>
@@ -12315,28 +12315,28 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
+          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
+          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
         </is>
       </c>
       <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
+          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
+          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
         </is>
       </c>
     </row>
@@ -12348,94 +12348,94 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
+          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
+          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
         </is>
       </c>
       <c r="D361" t="inlineStr"/>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
+          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>photo, top-news</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
+          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
         </is>
       </c>
       <c r="D362" t="inlineStr"/>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
+          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
+          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>photo, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
+          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
         </is>
       </c>
       <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
+          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
+          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
         </is>
       </c>
     </row>
@@ -12447,28 +12447,28 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
+          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
+          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
         </is>
       </c>
       <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
+          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
         </is>
       </c>
     </row>
@@ -12480,28 +12480,28 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
+          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
+          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
         </is>
       </c>
       <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
+          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12513,28 +12513,28 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
+          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
+          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
         </is>
       </c>
       <c r="D366" t="inlineStr"/>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
+          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
+          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12546,28 +12546,28 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
+          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
+          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
         </is>
       </c>
       <c r="D367" t="inlineStr"/>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
+          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
+          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
         </is>
       </c>
     </row>
@@ -12579,28 +12579,28 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
+          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
+          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
         </is>
       </c>
       <c r="D368" t="inlineStr"/>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
+          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
         </is>
       </c>
     </row>
@@ -12612,28 +12612,28 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
+          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
+          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
         </is>
       </c>
       <c r="D369" t="inlineStr"/>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
+          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12645,28 +12645,28 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
+          <t>Aktor senior Diding Boneng meninggal dunia</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
+          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
         </is>
       </c>
       <c r="D370" t="inlineStr"/>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
+          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
+          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12678,28 +12678,28 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Aktor senior Diding Boneng meninggal dunia</t>
+          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
+          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
         </is>
       </c>
       <c r="D371" t="inlineStr"/>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
+          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12711,28 +12711,28 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
+          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
+          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
         </is>
       </c>
       <c r="D372" t="inlineStr"/>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
+          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
+          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12744,28 +12744,28 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
+          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
+          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
         </is>
       </c>
       <c r="D373" t="inlineStr"/>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
+          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
         </is>
       </c>
     </row>
@@ -12777,28 +12777,28 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
+          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
+          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
         </is>
       </c>
       <c r="D374" t="inlineStr"/>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
+          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
+          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12810,28 +12810,28 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
+          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
+          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
         </is>
       </c>
       <c r="D375" t="inlineStr"/>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
+          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
         </is>
       </c>
     </row>
@@ -12843,28 +12843,28 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
+          <t>Harga bensin turun pada pekan pertama Agustus</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
+          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
         </is>
       </c>
       <c r="D376" t="inlineStr"/>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
+          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
+          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
         </is>
       </c>
     </row>
@@ -12876,61 +12876,61 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Harga bensin turun pada pekan pertama Agustus</t>
+          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
+          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
         </is>
       </c>
       <c r="D377" t="inlineStr"/>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
+          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
+          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
+          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
+          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
         </is>
       </c>
       <c r="D378" t="inlineStr"/>
       <c r="E378" t="inlineStr">
         <is>
-          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
+          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
+          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
         </is>
       </c>
     </row>
@@ -12942,28 +12942,28 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
+          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
+          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
         </is>
       </c>
       <c r="D379" t="inlineStr"/>
       <c r="E379" t="inlineStr">
         <is>
-          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
+          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
+          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
         </is>
       </c>
     </row>
@@ -12975,28 +12975,28 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
+          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
+          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
         </is>
       </c>
       <c r="D380" t="inlineStr"/>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
+          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
+          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
         </is>
       </c>
     </row>
@@ -13008,28 +13008,28 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
+          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
+          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
         </is>
       </c>
       <c r="D381" t="inlineStr"/>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
+          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
         </is>
       </c>
     </row>
@@ -13041,28 +13041,28 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
+          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
+          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
         </is>
       </c>
       <c r="D382" t="inlineStr"/>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
+          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
+          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
         </is>
       </c>
     </row>
@@ -13074,28 +13074,28 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
+          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
+          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
         </is>
       </c>
       <c r="D383" t="inlineStr"/>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
+          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
         </is>
       </c>
     </row>
@@ -13107,28 +13107,28 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
+          <t>Menjaga pintu air perekonomian Indonesia</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
+          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
         </is>
       </c>
       <c r="D384" t="inlineStr"/>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
+          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
+          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
         </is>
       </c>
     </row>
@@ -13140,28 +13140,28 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Menjaga pintu air perekonomian Indonesia</t>
+          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
+          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
         </is>
       </c>
       <c r="D385" t="inlineStr"/>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
+          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
         </is>
       </c>
     </row>
@@ -13173,28 +13173,28 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
+          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
+          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
         </is>
       </c>
       <c r="D386" t="inlineStr"/>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
+          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
+          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
         </is>
       </c>
     </row>
@@ -13206,28 +13206,28 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
+          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
+          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
         </is>
       </c>
       <c r="D387" t="inlineStr"/>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
+          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
         </is>
       </c>
     </row>
@@ -13239,61 +13239,61 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
+          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
+          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
         </is>
       </c>
       <c r="D388" t="inlineStr"/>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
+          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
+          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
+          <t>Kementerian ATR/BPN telah terbitkan 124 ribu SK sertifikat rumah MBR</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
+          <t>Mon, 03 Aug 2026 22:56:36 +0700</t>
         </is>
       </c>
       <c r="D389" t="inlineStr"/>
       <c r="E389" t="inlineStr">
         <is>
-          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
+          <t>Kementerian Agraria dan Tata Ruang/Badan Pertanahan Nasional (ATR/BPN) menyatakan telah menerbitkan surat keputusan ...</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5678484/kementerian-atr-bpn-telah-terbitkan-124-ribu-sk-sertifikat-rumah-mbr</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_224532.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update berita 2026-08-03 22:51 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-08-03.xlsx
+++ b/data/berita_antara_2026-08-03.xlsx
@@ -11159,28 +11159,28 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
+          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
+          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
         </is>
       </c>
       <c r="D325" t="inlineStr"/>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
+          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
+          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
         </is>
       </c>
     </row>
@@ -11192,28 +11192,28 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
+          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
+          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
         </is>
       </c>
       <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
+          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
+          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
         </is>
       </c>
     </row>
@@ -11225,61 +11225,61 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
+          <t>Chelsea umumkan transfer gelandang Inggris Jordan Henderson</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
+          <t>Mon, 03 Aug 2026 23:59:34 +0700</t>
         </is>
       </c>
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr">
         <is>
-          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
+          <t>Chelsea resmi mengumumkan kedatangan gelandang senior asal Inggris Jordan Henderson dengan status bebas transfer ...</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
+          <t>https://www.antaranews.com/berita/5678548/chelsea-umumkan-transfer-gelandang-inggris-jordan-henderson</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000042505.jpg</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
+          <t>Nguyen Xuan Son ungkap alasan tak jadi starter saat kalahkan Indonesia</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:56:45 +0700</t>
         </is>
       </c>
       <c r="D328" t="inlineStr"/>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
+          <t>Penyerang Timnas Vietnam Nguyen Xuan Son mengungkapkan alasan dirinya tidak dimainkan sebagai starter saat timnya ...</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
+          <t>https://www.antaranews.com/berita/5678547/nguyen-xuan-son-ungkap-alasan-tak-jadi-starter-saat-kalahkan-indonesia</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1003314030.jpg</t>
         </is>
       </c>
     </row>
@@ -11291,28 +11291,28 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
+          <t>Indonesia-Thailand sepakati penguatan kerja sama lintas bidang</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:55:47 +0700</t>
         </is>
       </c>
       <c r="D329" t="inlineStr"/>
       <c r="E329" t="inlineStr">
         <is>
-          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
+          <t>ANTARA - Indonesia dan Thailand sepakat memperkuat kemitraan strategis di berbagai sektor, mulai dari keamanan, ...</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
+          <t>https://www.antaranews.com/video/5678533/indonesia-thailand-sepakati-penguatan-kerja-sama-lintas-bidang</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/INDONESIA-THAILAND-SEPAKATI-PENGUATAN-KERJA-SAMA-LINTAS-BIDANG.jpg</t>
         </is>
       </c>
     </row>
@@ -11324,61 +11324,61 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
+          <t>BPS kaitkan kenaikan TPK hotel bintang dengan kualitas wisman</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
+          <t>Mon, 03 Aug 2026 23:53:51 +0700</t>
         </is>
       </c>
       <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
+          <t>Badan Pusat Statistik (BPS) Bali mengaitkan kenaikan tingkat penghunian kamar (TPK) hotel bintang pada Juni 2026 dengan ...</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
+          <t>https://www.antaranews.com/berita/5678543/bps-kaitkan-kenaikan-tpk-hotel-bintang-dengan-kualitas-wisman</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0332.jpeg</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
+          <t>Jogja Run'nShine 2026 targetkan diikuti 3.500 pelari</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
+          <t>Mon, 03 Aug 2026 23:52:29 +0700</t>
         </is>
       </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
+          <t>Pergelaran Jogja Run'nShine 2026 menargetkan diikuti sebanyak 3.500 pelari dengan memberikan pengalaman konsep ...</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
+          <t>https://www.antaranews.com/berita/5678540/jogja-runnshine-2026-targetkan-diikuti-3500-pelari</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0103.jpg</t>
         </is>
       </c>
     </row>
@@ -11390,61 +11390,61 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
+          <t>Jenama perkakas otomotif Tekiro dapat pengakuan Guinnes World Records</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
+          <t>Mon, 03 Aug 2026 23:47:06 +0700</t>
         </is>
       </c>
       <c r="D332" t="inlineStr"/>
       <c r="E332" t="inlineStr">
         <is>
-          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
+          <t>Jenama perkakas otomotif Tekiro mendapat pengakuan dari Guiness World Records berkat ...</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
+          <t>https://otomotif.antaranews.com/berita/5678535/jenama-perkakas-otomotif-tekiro-dapat-pengakuan-guinnes-world-records</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-02-at-15.34.09-1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
+          <t>Pemkab Sleman dukung kejuaraan dragbike tingkatkan ekonomi masyarakat</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
+          <t>Mon, 03 Aug 2026 23:42:42 +0700</t>
         </is>
       </c>
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
+          <t>Pemerintah Kabupaten Sleman, Daerah Istimewa Yogyakarta, mendukung penuh penyelenggaraan Kejuaraan Dragbike Super ...</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
+          <t>https://www.antaranews.com/berita/5678532/pemkab-sleman-dukung-kejuaraan-dragbike-tingkatkan-ekonomi-masyarakat</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000029422.jpg</t>
         </is>
       </c>
     </row>
@@ -11456,28 +11456,28 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
+          <t>GMR nilai akses penerbangan langsung buka peluang ekonomi RI-India</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
+          <t>Mon, 03 Aug 2026 23:41:32 +0700</t>
         </is>
       </c>
       <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr">
         <is>
-          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
+          <t>GMR Group, perusahaan multinasional India yang bergerak di bidang infrastruktur, menilai akses penerbangan langsung ...</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
+          <t>https://www.antaranews.com/berita/5678529/gmr-nilai-akses-penerbangan-langsung-buka-peluang-ekonomi-ri-india</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/DSF3021.jpeg</t>
         </is>
       </c>
     </row>
@@ -11489,94 +11489,94 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
+          <t>PSSI raup dana Rp722 miliar dalam laporan keuangan tahunan</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
+          <t>Mon, 03 Aug 2026 23:37:46 +0700</t>
         </is>
       </c>
       <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
+          <t>Ketua Umum Persatuan Sepak Bola Seluruh Indonesia (PSSI) Erick Thohir menyebut organisasinya meraup dana senilai Rp722 ...</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
+          <t>https://www.antaranews.com/berita/5678528/pssi-raup-dana-rp722-miliar-dalam-laporan-keuangan-tahunan</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0098_1.jpg</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
+          <t>Otorita kolaborasi PNM untuk pengembangan ekonomi masyarakat IKN</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:50 +0700</t>
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
       <c r="E336" t="inlineStr">
         <is>
-          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
+          <t>Otorita Ibu Kota Nusantara (IKN) melakukan kolaborasi dengan PT Permodalan Nasional Madani (Persero) untuk pengembangan ...</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
+          <t>https://www.antaranews.com/berita/5678525/otorita-kolaborasi-pnm-untuk-pengembangan-ekonomi-masyarakat-ikn</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0012_1.jpg</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
+          <t>DPR: Wacana Prabowo jembatani dialog Korea sesuai politik bebas aktif</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:13 +0700</t>
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
       <c r="E337" t="inlineStr">
         <is>
-          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
+          <t>Wakil Ketua Komisi I DPR RI Dave Laksono menilai wacana Presiden Prabowo Subianto untuk menjembatani dialog antara ...</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
+          <t>https://www.antaranews.com/berita/5678521/dpr-wacana-prabowo-jembatani-dialog-korea-sesuai-politik-bebas-aktif</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/22/IMG_20260422_175322.jpg</t>
         </is>
       </c>
     </row>
@@ -11588,193 +11588,193 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
+          <t>Kongres PSSI sepakati pemilihan pengurus mundur ke Juli 2027</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
+          <t>Mon, 03 Aug 2026 23:30:00 +0700</t>
         </is>
       </c>
       <c r="D338" t="inlineStr"/>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
+          <t>ANTARA - Kongres Biasa PSSI 2026 menyepakati perubahan jadwal Kongres Pemilihan Pengurus PSSI 2027 dari semula Mei ...</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
+          <t>https://www.antaranews.com/video/5678395/kongres-pssi-sepakati-pemilihan-pengurus-mundur-ke-juli-2027</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KONGRES-PSSI-SEPAKATI-PEMILIHAN-PENGURUS-MUNDUR-KE-JULI-2027.jpg</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
+          <t>Toyota Astra Motor perkenalkan Hilux generasi ke-9</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:25:20 +0700</t>
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
+          <t>PT Toyota Astra Motor (TAM) memperkenalkan Hilux generasi ke-9 untuk mendukung pemenuhan kebutuhan operasional industri ...</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
+          <t>https://otomotif.antaranews.com/berita/5678519/toyota-astra-motor-perkenalkan-hilux-generasi-ke-9</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/photo_6307309656757440820_w-1.jpg</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
+          <t>Sudin PPAPP Jakbar sosialisasikan Sekolah Siaga Kependudukan</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:24:33 +0700</t>
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
+          <t>Suku Dinas Pemberdayaan, Perlindungan Anak, dan Pengendalian Penduduk (Sudin PPAPP) Jakarta Barat (Jakbar) menggelar ...</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
+          <t>https://www.antaranews.com/berita/5678515/sudin-ppapp-jakbar-sosialisasikan-sekolah-siaga-kependudukan</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0031_1.jpg</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
+          <t>Klasemen Grup A Piala AFF : Timnas Indonesia turun ke peringkat tiga</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:51 +0700</t>
         </is>
       </c>
       <c r="D341" t="inlineStr"/>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
+          <t>Timnas Indonesia turun ke peringkat ketiga klasemen sementara Grup A Piala AFF 2026 setelah menelan kekalahan 0-3 dari ...</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
+          <t>https://www.antaranews.com/berita/5678512/klasemen-grup-a-piala-aff-timnas-indonesia-turun-ke-peringkat-tiga</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/timnas-indonesia-lawan-vietnam-di-piala-aff-2833516.jpg</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
+          <t>NTB menargetkan penonton MotoGP Mandalika tembus 140 ribu</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
+          <t>Mon, 03 Aug 2026 23:23:01 +0700</t>
         </is>
       </c>
       <c r="D342" t="inlineStr"/>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
+          <t>Pemerintah Provinsi Nusa Tenggara Barat menargetkan jumlah penonton MotoGP di Sirkuit Mandalika pada 9-11 Oktober 2026 ...</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
+          <t>https://www.antaranews.com/berita/5678508/ntb-menargetkan-penonton-motogp-mandalika-tembus-140-ribu</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260109-WA0024_copy_1280x797.jpg</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>ekonomi-bisnis, terkini</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
+          <t>Bulog: Margin naik jadi 7 persen, dukungan Presiden kawal swasembada</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
+          <t>Mon, 03 Aug 2026 23:19:51 +0700</t>
         </is>
       </c>
       <c r="D343" t="inlineStr"/>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
+          <t>Direktur Utama Perum Bulog Ahmad Rizal Ramdhani menegaskan kenaikan margin fee menjadi 7 persen bentuk dukungan ...</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
+          <t>https://www.antaranews.com/berita/5678504/bulog-margin-naik-jadi-7-persen-dukungan-presiden-kawal-swasembada</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/14C1B7CB-9D6F-49B9-9CD1-E40DD76E851C.jpeg</t>
         </is>
       </c>
     </row>
@@ -11786,28 +11786,28 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
+          <t>Turkiye sebut serangan Israel sabotase upaya damai di Gaza</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
+          <t>Mon, 03 Aug 2026 23:18:30 +0700</t>
         </is>
       </c>
       <c r="D344" t="inlineStr"/>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
+          <t>Pemerintah Turkiye pada Senin menilai serangan Israel di Jalur Gaza telah menghambat berbagai inisiatif diplomatik yang ...</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
+          <t>https://www.antaranews.com/berita/5678500/turkiye-sebut-serangan-israel-sabotase-upaya-damai-di-gaza</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/thumbs_b_c_186832d7ab4775afec853057c8952c3d.jpg</t>
         </is>
       </c>
     </row>
@@ -11819,94 +11819,94 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Kemenbud hadirkan GBN untuk membina talenta seni musik nasional</t>
+          <t>Purbaya pastikan tak ada lagi perdebatan soal penarikan SAL dari bank</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:07:01 +0700</t>
+          <t>Mon, 03 Aug 2026 23:15:59 +0700</t>
         </is>
       </c>
       <c r="D345" t="inlineStr"/>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Kementerian Kebudayaan (Kemenbud) menghadirkan program pembinaan talenta seni musik nasional yang mempertemukan ...</t>
+          <t>Menteri Keuangan (Menkeu), Purbaya Yudhi Sadewa memastikan tidak ada lagi perdebatan mengenai penarikan dana ...</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678491/kemenbud-hadirkan-gbn-untuk-membina-talenta-seni-musik-nasional</t>
+          <t>https://www.antaranews.com/berita/5678499/purbaya-pastikan-tak-ada-lagi-perdebatan-soal-penarikan-sal-dari-bank</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.28.05.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-23.02.47.jpeg</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>ekonomi-bisnis, terkini</t>
+          <t>terkini</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
+          <t>Tim 9 Kejagung didesak usut pemilik uang-emas di rumah eks Jampidsus</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
+          <t>Mon, 03 Aug 2026 23:10:43 +0700</t>
         </is>
       </c>
       <c r="D346" t="inlineStr"/>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
+          <t>Tim 9 Kejaksaan Agung didesak mengusut tuntas pemilik uang tunai senilai Rp476 miliar dan emas batangan seberat 74 ...</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
+          <t>https://www.antaranews.com/berita/5678495/tim-9-kejagung-didesak-usut-pemilik-uang-emas-di-rumah-eks-jampidsus</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/1000175632.jpg</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>terkini</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>PBSI buka suara soal absennya Jafar/Felisha di Kejuaraan Dunia BWF</t>
+          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 23:03:05 +0700</t>
+          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
         </is>
       </c>
       <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr">
         <is>
-          <t>Pengurus Pusat PBSI menyatakan absennya dua pasangan ganda campuran Indonesia Jafar Hidayatullah/Felisha Alberta ...</t>
+          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678487/pbsi-buka-suara-soal-absennya-jafar-felisha-di-kejuaraan-dunia-bwf</t>
+          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/03/06/IMG_20251127_205351.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
         </is>
       </c>
     </row>
@@ -11918,160 +11918,160 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Prabowo terima tanda kehormatan dari Angkatan Bersenjata Thailand</t>
+          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:59:35 +0700</t>
+          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
         </is>
       </c>
       <c r="D348" t="inlineStr"/>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto menerima tanda kehormatan dari Angkatan Bersenjata Kerajaan Thailand yang diberikan pada saat ...</t>
+          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678283/prabowo-terima-tanda-kehormatan-dari-angkatan-bersenjata-thailand</t>
+          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/tempImageNOyDfK.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Indonesia punya 2.723 warisan budaya, Menbud: jaga untuk wisata budaya</t>
+          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:50:37 +0700</t>
+          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
         </is>
       </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr">
         <is>
-          <t>ANTARA - Menteri Kebudayaan, Fadli Zon, Senin (3/8), menekankan pengembangan wisata budaya di setiap daerah bahkan ...</t>
+          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678243/indonesia-punya-2723-warisan-budaya-menbud-jaga-untuk-wisata-budaya</t>
+          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_INDONESIA-PUNYA-2.723-WARISAN-BUDAYA-MENBUD-JAGA-UNTUK-WISATA-BUDAYA.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Menkeu: Eskalasi konflik Timteng dorong imbal hasil SBN ke 7,14 persen</t>
+          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 20:48:02 +0700</t>
+          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
         </is>
       </c>
       <c r="D350" t="inlineStr"/>
       <c r="E350" t="inlineStr">
         <is>
-          <t>Menteri Keuangan Purbaya Yudhi Sadewa mengatakan eskalasi konflik di Timur Tengah mendorong kenaikan imbal hasil Surat ...</t>
+          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678253/menkeu-eskalasi-konflik-timteng-dorong-imbal-hasil-sbn-ke-714-persen</t>
+          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-20.38.31.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial, top-news</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Prabowo dukung peningkatan latihan bersama militer RI-Thailand</t>
+          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:21:32 +0700</t>
+          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
         </is>
       </c>
       <c r="D351" t="inlineStr"/>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto mendukung peningkatan frekuensi latihan bersama antara Tentara Nasional Indonesia (TNI) dan ...</t>
+          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678081/prabowo-dukung-peningkatan-latihan-bersama-militer-ri-thailand</t>
+          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.41.07.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>ekonomi-finansial, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>OJK: Kredit perbankan tumbuh 12,67 persen capai Rp9.080,9 triliun</t>
+          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:12:24 +0700</t>
+          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
         </is>
       </c>
       <c r="D352" t="inlineStr"/>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Otoritas Jasa Keuangan (OJK) melaporkan penyaluran kredit perbankan di tanah air tumbuh 12,67 persen year on year ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678057/ojk-kredit-perbankan-tumbuh-1267-persen-capai-rp90809-triliun</t>
+          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.15.18_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
         </is>
       </c>
     </row>
@@ -12083,28 +12083,28 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Menkomdigi: KIP garda depan informasi jernih dan perangi hoaks</t>
+          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 19:00:50 +0700</t>
+          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
         </is>
       </c>
       <c r="D353" t="inlineStr"/>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid mengatakan Komisi Informasi Pusat (KIP) menjadi garda terdepan ...</t>
+          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678033/menkomdigi-kip-garda-depan-informasi-jernih-dan-perangi-hoaks</t>
+          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0321.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
         </is>
       </c>
     </row>
@@ -12116,28 +12116,28 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Satu tahun Sekolah Rakyat, ratusan siswa torehkan prestasi</t>
+          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:59:25 +0700</t>
+          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
         </is>
       </c>
       <c r="D354" t="inlineStr"/>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Menteri Sosial (Mensos) Saifullah Yusuf menyatakan selama satu tahun Sekolah Rakyat berdiri sudah ratusan ...</t>
+          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678024/satu-tahun-sekolah-rakyat-ratusan-siswa-torehkan-prestasi</t>
+          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000176441.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
         </is>
       </c>
     </row>
@@ -12149,28 +12149,28 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Menkeu: Realisasi anggaran MBG Rp101,1 T untuk 63,13 juta penerima</t>
+          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:53:14 +0700</t>
+          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
         </is>
       </c>
       <c r="D355" t="inlineStr"/>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Menteri Keuangan (Menkeu) Purbaya Yudhi Sadewa mengungkapkan bahwa realisasi anggaran Program Makan Bergizi Gratis ...</t>
+          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678005/menkeu-realisasi-anggaran-mbg-rp1011-t-untuk-6313-juta-penerima</t>
+          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29-2.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
         </is>
       </c>
     </row>
@@ -12182,28 +12182,28 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Polri perkuat langkah preventif respons isu keamanan nasional</t>
+          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:46:34 +0700</t>
+          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
         </is>
       </c>
       <c r="D356" t="inlineStr"/>
       <c r="E356" t="inlineStr">
         <is>
-          <t>Polri memastikan terus memperkuat langkah preventif untuk menjaga keamanan nasional sehingga aktivitas masyarakat dan ...</t>
+          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677985/polri-perkuat-langkah-preventif-respons-isu-keamanan-nasional</t>
+          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/1000086556.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
         </is>
       </c>
     </row>
@@ -12215,28 +12215,29 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Prabowo dan PM Thailand bertemu empat mata di Istana Merdeka</t>
+          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:49:52 +0700</t>
+          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
         </is>
       </c>
       <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr">
         <is>
-          <t>Presiden Prabowo Subianto dan Perdana Menteri Thailand Anutin Charnvirakul menggelar pertemuan empat mata di Istana ...</t>
+          <t>nya tidak dilanjutkan," ucap Sudaryono.
+Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677828/prabowo-dan-pm-thailand-bertemu-empat-mata-di-istana-merdeka</t>
+          <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_5162.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
         </is>
       </c>
     </row>
@@ -12248,29 +12249,28 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Kepala BGN tingkatkan status keracunan MBG jadi kejadian fatal</t>
+          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:10:19 +0700</t>
+          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
         </is>
       </c>
       <c r="D358" t="inlineStr"/>
       <c r="E358" t="inlineStr">
         <is>
-          <t>nya tidak dilanjutkan," ucap Sudaryono.
-Ia menegaskan BGN memberlakukan nol toleransi pada setiap status ...</t>
+          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677743/kepala-bgn-tingkatkan-status-keracunan-mbg-jadi-kejadian-fatal</t>
+          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/01/ZAM02548_edit_2028523819372755.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
         </is>
       </c>
     </row>
@@ -12282,28 +12282,28 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Harga minyak turun usai AS siap lanjutkan dialog dengan Iran</t>
+          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 17:08:35 +0700</t>
+          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
         </is>
       </c>
       <c r="D359" t="inlineStr"/>
       <c r="E359" t="inlineStr">
         <is>
-          <t>Harga minyak turun lebih dari 5 persen, Senin, setelah Presiden Amerika Serikat Donald Trump ...</t>
+          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677735/harga-minyak-turun-usai-as-siap-lanjutkan-dialog-dengan-iran</t>
+          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/ilustrasi-isi-bensin-di-pom.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
         </is>
       </c>
     </row>
@@ -12315,94 +12315,94 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Australia konfirmasi kematian massal pertama satwa akibat flu burung</t>
+          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:48:50 +0700</t>
+          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
         </is>
       </c>
       <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Australia mengonfirmasi kematian massal satwa liar pertama terkait flu burung H5 yang mematikan, dengan burung camar ...</t>
+          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677701/australia-konfirmasi-kematian-massal-pertama-satwa-akibat-flu-burung</t>
+          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/06/26/Virus-flu-burung-penyakit-unggas.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>photo, top-news</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Siklon 94 W,  waspada cuaca ekstrem &amp; gelombang tinggi di wilayah RI</t>
+          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:30:38 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
         </is>
       </c>
       <c r="D361" t="inlineStr"/>
       <c r="E361" t="inlineStr">
         <is>
-          <t>Badan Meteorologi, Klimatologi, dan Geofisika (BMKG) mendeteksi pergerakan Bibit Siklon Tropis 94W di Laut Filipina ...</t>
+          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677641/siklon-94-w-waspada-cuaca-ekstrem-gelombang-tinggi-di-wilayah-ri</t>
+          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/27/1000395034.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>photo, top-news</t>
+          <t>top-news</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Petani berbagi air sumur demi selamatkan tanaman tembakau</t>
+          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:51 +0700</t>
+          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
         </is>
       </c>
       <c r="D362" t="inlineStr"/>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Petani mengambil air dari sumur untuk menyiram tanaman tembakau di Lengkong, Nganjuk, Jawa Timur, Senin (3/8/2026). ...</t>
+          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/foto/5677428/petani-berbagi-air-sumur-demi-selamatkan-tanaman-tembakau</t>
+          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/petani-tembakau-berbagi-air-sumur-antisipasi-dampak-el-nino-030826-mm-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
         </is>
       </c>
     </row>
@@ -12414,28 +12414,28 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Nusron sebut banyak laut di Batam telah dikapling tanpa prosedur sah</t>
+          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:44:05 +0700</t>
+          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
         </is>
       </c>
       <c r="D363" t="inlineStr"/>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Menteri Agraria dan Tata Ruang (ATR)/Kepala Badan Pertanahan Nasional (BPN) Nusron Wahid mengatakan, menerima banyak ...</t>
+          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677425/nusron-sebut-banyak-laut-di-batam-telah-dikapling-tanpa-prosedur-sah</t>
+          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_142345.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
         </is>
       </c>
     </row>
@@ -12447,28 +12447,28 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Menkomdigi panggil YouTube imbas temuan konten promosi vape sasar anak</t>
+          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 14:22:09 +0700</t>
+          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
         </is>
       </c>
       <c r="D364" t="inlineStr"/>
       <c r="E364" t="inlineStr">
         <is>
-          <t>Menteri Komunikasi dan Digital (Menkomdigi) Meutya Hafid merencanakan pemanggilan terhadap platform digital YouTube ...</t>
+          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677396/menkomdigi-panggil-youtube-imbas-temuan-konten-promosi-vape-sasar-anak</t>
+          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG-20260803-WA0225.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12480,28 +12480,28 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Kemnaker: Magang Nasional diharapkan menekan angka pengangguran muda</t>
+          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:37:57 +0700</t>
+          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
         </is>
       </c>
       <c r="D365" t="inlineStr"/>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Kementerian Ketenagakerjaan (Kemnaker) mengatakan program Magang Nasional (MagangHub) untuk mempersiapkan kompetensi ...</t>
+          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677364/kemnaker-magang-nasional-diharapkan-menekan-angka-pengangguran-muda</t>
+          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/04/23/ff63afaf-7778-47fe-833d-5a8068af9a51_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12513,28 +12513,28 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Kemenag perkuat transformasi madrasah lewat revitalisasi-digitalisasi</t>
+          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:36:36 +0700</t>
+          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
         </is>
       </c>
       <c r="D366" t="inlineStr"/>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Menteri Agama (Menag) Nasaruddin Umar menegaskan transformasi madrasah terus diperkuat melalui revitalisasi ...</t>
+          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677363/kemenag-perkuat-transformasi-madrasah-lewat-revitalisasi-digitalisasi</t>
+          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/14/1000173935_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
         </is>
       </c>
     </row>
@@ -12546,28 +12546,28 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Lisensi IP Global Buka Peluang Bisnis Baru bagi Kreator Indonesia</t>
+          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:34:30 +0700</t>
+          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
         </is>
       </c>
       <c r="D367" t="inlineStr"/>
       <c r="E367" t="inlineStr">
         <is>
-          <t>Wakil Menteri Ekonomi Kreatif Irene Umar mengatakan kolaborasi antara pemilik kekayaan intelektual (Intellectual ...</t>
+          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677353/lisensi-ip-global-buka-peluang-bisnis-baru-bagi-kreator-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000589873.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
         </is>
       </c>
     </row>
@@ -12579,28 +12579,28 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Nilai ekspor perdagangan RI Januari-Juni capai 140,81 miliar dolar AS</t>
+          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:16:17 +0700</t>
+          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
         </is>
       </c>
       <c r="D368" t="inlineStr"/>
       <c r="E368" t="inlineStr">
         <is>
-          <t>Badan Pusat Statistik (BPS) mencatat nilai ekspor Indonesia secara kumulatif dari Januari-Juni 2026 mencapai 140,81 ...</t>
+          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677315/nilai-ekspor-perdagangan-ri-januari-juni-capai-14081-miliar-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/02/neraca-perdagangan-januari-mei-2026-surplus-2815779.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12612,28 +12612,28 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Korban KMP Mutiara Sentosa II dievakuasi ke Pelabuhan Tanjung Perak</t>
+          <t>Aktor senior Diding Boneng meninggal dunia</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 13:06:15 +0700</t>
+          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
         </is>
       </c>
       <c r="D369" t="inlineStr"/>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Tim SAR gabungan terus melakukan evakuasi korban terbakarnya KMP Mutiara Sentosa 2 ke darat, tepatnya ke Pelabuhan ...</t>
+          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677297/korban-kmp-mutiara-sentosa-ii-dievakuasi-ke-pelabuhan-tanjung-perak</t>
+          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/260821_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12645,28 +12645,28 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Aktor senior Diding Boneng meninggal dunia</t>
+          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:39:03 +0700</t>
+          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
         </is>
       </c>
       <c r="D370" t="inlineStr"/>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Aktor sekaligus komedian tanah air, Zainal Abidin alias Diding Boneng dikabarkan meninggal dunia pada Senin (3/8) dalam ...</t>
+          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677209/aktor-senior-diding-boneng-meninggal-dunia</t>
+          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/26f1eb88-3301-4ae1-badd-bed5078fe3dd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
         </is>
       </c>
     </row>
@@ -12678,28 +12678,28 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Seskab: Prabowo dorong sinergi pemerintah dan dunia usaha</t>
+          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 11:17:50 +0700</t>
+          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
         </is>
       </c>
       <c r="D371" t="inlineStr"/>
       <c r="E371" t="inlineStr">
         <is>
-          <t>Sekretaris Kabinet Teddy Indra Wijaya menyampaikan bahwa Presiden Prabowo Subianto menekankan pentingnya sinergi antara ...</t>
+          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677191/seskab-prabowo-dorong-sinergi-pemerintah-dan-dunia-usaha</t>
+          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_0891_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
         </is>
       </c>
     </row>
@@ -12711,28 +12711,28 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>Red Velvet bersiap kembali lewat EP baru "Velvet Summer"</t>
+          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:24:37 +0700</t>
+          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
         </is>
       </c>
       <c r="D372" t="inlineStr"/>
       <c r="E372" t="inlineStr">
         <is>
-          <t>Grup idola K-pop Red Velvet akan kembali lewat rilis mini album atau extended play (EP) baru bertajuk “Velvet ...</t>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677151/red-velvet-bersiap-kembali-lewat-ep-baru-velvet-summer</t>
+          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/ca97a3a8-aa17-45fc-be71-d36051dd9dcd.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
         </is>
       </c>
     </row>
@@ -12744,28 +12744,28 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Menaker pastikan komitmen pemerintah perkuat kesejahteraan pekerja</t>
+          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:16:19 +0700</t>
+          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
         </is>
       </c>
       <c r="D373" t="inlineStr"/>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Menteri Ketenagakerjaan (Menaker) Yassierli memastikan pemerintah berkomitmen untuk memperkuat kesejahteraan, ...</t>
+          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677148/menaker-pastikan-komitmen-pemerintah-perkuat-kesejahteraan-pekerja</t>
+          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/09/20/pelepasan-peserta-pemagangan-ke-jepang-di-jawa-barat-2627513.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
         </is>
       </c>
     </row>
@@ -12777,28 +12777,28 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>23 calon hakim agung dan ad hoc ikuti seleksi wawancara akhir</t>
+          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:15:01 +0700</t>
+          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
         </is>
       </c>
       <c r="D374" t="inlineStr"/>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Sebanyak 23 orang calon hakim agung dan ad hoc Mahkamah Agung Tahun 2026 mengikuti seleksi wawancara tahap akhir di ...</t>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677137/23-calon-hakim-agung-dan-ad-hoc-ikuti-seleksi-wawancara-akhir</t>
+          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1000012883_1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
         </is>
       </c>
     </row>
@@ -12810,28 +12810,28 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>BRIN perkuat kajian sungai bawah tanah di Kebumen untuk ketahanan air</t>
+          <t>Harga bensin turun pada pekan pertama Agustus</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:57:19 +0700</t>
+          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
         </is>
       </c>
       <c r="D375" t="inlineStr"/>
       <c r="E375" t="inlineStr">
         <is>
-          <t>Badan Riset dan Inovasi Nasional (BRIN) memperkuat riset ketahanan air melalui pengembangan teknologi dan penelitian ...</t>
+          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677120/brin-perkuat-kajian-sungai-bawah-tanah-di-kebumen-untuk-ketahanan-air</t>
+          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/1785706440-47672950-1.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
         </is>
       </c>
     </row>
@@ -12843,61 +12843,61 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Harga bensin turun pada pekan pertama Agustus</t>
+          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:51:00 +0700</t>
+          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
         </is>
       </c>
       <c r="D376" t="inlineStr"/>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Harga bahan bakar minyak (BBM) jenis bensin di stasiun pengisian bahan bakar umum (SPBU) Pertamina, Shell, dan bp ...</t>
+          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677109/harga-bensin-turun-pada-pekan-pertama-agustus</t>
+          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2024/10/02/penuruanan-harga-bbm-011024-aaa-7.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>top-news</t>
+          <t>ekonomi-finansial</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Sean Gelael berbagi pengalaman di dunia balap ke pengunjung GIIAS 2026</t>
+          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:34:53 +0700</t>
+          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
         </is>
       </c>
       <c r="D377" t="inlineStr"/>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Pembalap Indonesia Sean Gelael berbagi pengalamannya di dunia balap ke pengunjung GAIKINDO Indonesia International ...</t>
+          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677103/sean-gelael-berbagi-pengalaman-di-dunia-balap-ke-pengunjung-giias-2026</t>
+          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/16b70b87-326f-479a-a806-580ab846cc6f_1.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
         </is>
       </c>
     </row>
@@ -12909,28 +12909,28 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Cadangan devisa RI jadi 145 M dolar AS, BI sebut masih di level aman</t>
+          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:52:44 +0700</t>
+          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
         </is>
       </c>
       <c r="D378" t="inlineStr"/>
       <c r="E378" t="inlineStr">
         <is>
-          <t>ANTARA - Bank Indonesia (BI) mengungkapkan cadangan devisa pada akhir Juli 2026 berada di posisi 145 miliar dolar AS. ...</t>
+          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/video/5678347/cadangan-devisa-ri-jadi-145-m-dolar-as-bi-sebut-masih-di-level-aman</t>
+          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AB_CADANGAN-DEVISA-RI-JADI-145-M-DOLAR-AS-BI-SEBUT-MASIH-DI-LEVEL-AMAN.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
         </is>
       </c>
     </row>
@@ -12942,28 +12942,28 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>BI: Inflasi Juli terjaga berkat sinergi bank sentral dan pemerintah</t>
+          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:51:39 +0700</t>
+          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
         </is>
       </c>
       <c r="D379" t="inlineStr"/>
       <c r="E379" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) memandang inflasi Indeks Harga Konsumen (IHK) pada Juli 2026 tetap terjaga dalam sasaran target, ...</t>
+          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678380/bi-inflasi-juli-terjaga-berkat-sinergi-bank-sentral-dan-pemerintah</t>
+          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/WhatsApp-Image-2026-07-07-at-14.31.59_edited.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
         </is>
       </c>
     </row>
@@ -12975,28 +12975,28 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>BI: Kepemilikan SRBI oleh bank guna kelola likuiditas, bukan investasi</t>
+          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 21:35:49 +0700</t>
+          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
         </is>
       </c>
       <c r="D380" t="inlineStr"/>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Bank Indonesia (BI) menegaskan bahwa Sekuritas Rupiah Bank Indonesia (SRBI) ditujukan sebagai instrumen pengelolaan ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5678351/bi-kepemilikan-srbi-oleh-bank-guna-kelola-likuiditas-bukan-investasi</t>
+          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-21.22.00.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
         </is>
       </c>
     </row>
@@ -13008,28 +13008,28 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>KSSK prakirakan pertumbuhan ekonomi RI pada 2026 capai 5,6-6 persen</t>
+          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 18:28:16 +0700</t>
+          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
         </is>
       </c>
       <c r="D381" t="inlineStr"/>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) memprakirakan ekonomi Indonesia sepanjang 2026 tumbuh dalam kisaran ...</t>
+          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677935/kssk-prakirakan-pertumbuhan-ekonomi-ri-pada-2026-capai-56-6-persen</t>
+          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-18.19.55.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
         </is>
       </c>
     </row>
@@ -13041,28 +13041,28 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Rupiah menguat dipengaruhi PMI manufaktur Indonesia naik jadi 50,2</t>
+          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:58:46 +0700</t>
+          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
         </is>
       </c>
       <c r="D382" t="inlineStr"/>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah terhadap dolar AS pada penutupan perdagangan Senin, bergerak menguat 25 poin atau 0,14 persen ...</t>
+          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677712/rupiah-menguat-dipengaruhi-pmi-manufaktur-indonesia-naik-jadi-502</t>
+          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/05/12/nilai-tukar-rupiah-melemah-115-poin-2788415.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
         </is>
       </c>
     </row>
@@ -13074,28 +13074,28 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>KSSK: Sistem keuangan TW-II tetap terjaga di tengah konflik geopolitik</t>
+          <t>Menjaga pintu air perekonomian Indonesia</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:26:03 +0700</t>
+          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
         </is>
       </c>
       <c r="D383" t="inlineStr"/>
       <c r="E383" t="inlineStr">
         <is>
-          <t>Komite Stabilitas Sistem Keuangan (KSSK) menilai kondisi fiskal, moneter dan sektor keuangan selama triwulan II 2026 ...</t>
+          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677625/kssk-sistem-keuangan-tw-ii-tetap-terjaga-di-tengah-konflik-geopolitik</t>
+          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/WhatsApp-Image-2026-08-03-at-15.32.29.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
         </is>
       </c>
     </row>
@@ -13107,28 +13107,28 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Menjaga pintu air perekonomian Indonesia</t>
+          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 16:04:40 +0700</t>
+          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
         </is>
       </c>
       <c r="D384" t="inlineStr"/>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Bayangkan perekonomian Indonesia sebagai sebuah bendungan raksasa yang mengairi hamparan persawahan. Air yang mengalir ...</t>
+          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677565/menjaga-pintu-air-perekonomian-indonesia</t>
+          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/peringati-hari-bank-indonesia-doku-perkuat-ekosistem-pembayaran-2817675.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
         </is>
       </c>
     </row>
@@ -13140,28 +13140,28 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Rupiah diperkirakan menguat seiring AS batalkan rencana serang Iran</t>
+          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 10:12:26 +0700</t>
+          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
         </is>
       </c>
       <c r="D385" t="inlineStr"/>
       <c r="E385" t="inlineStr">
         <is>
-          <t>Analis Doo Financial Futures, Lukman Leong memperkirakan rupiah menguat seiring Amerika Serikat (AS) membatalkan ...</t>
+          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677132/rupiah-diperkirakan-menguat-seiring-as-batalkan-rencana-serang-iran</t>
+          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828847.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
         </is>
       </c>
     </row>
@@ -13173,28 +13173,28 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Rupiah pada Senin pagi melemah jadi Rp18.031 per dolar AS</t>
+          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 09:05:50 +0700</t>
+          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
         </is>
       </c>
       <c r="D386" t="inlineStr"/>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Nilai tukar rupiah pada Senin pagi bergerak melemah 9 poin atau 0,05 persen menjadi Rp18.031 per dolar AS dibandingkan ...</t>
+          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5677063/rupiah-pada-senin-pagi-melemah-jadi-rp18031-per-dolar-as</t>
+          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/nilai-tukar-rupiah-melemah-2828879.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
         </is>
       </c>
     </row>
@@ -13206,61 +13206,61 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Komisi XI: PFII peluang RI tangkap momentum perpindahan modal global</t>
+          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:53:34 +0700</t>
+          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
         </is>
       </c>
       <c r="D387" t="inlineStr"/>
       <c r="E387" t="inlineStr">
         <is>
-          <t>Wakil Ketua Komisi XI DPR RI Mohamad Hekal mengatakan percepatan pembentukan Pusat Finansial Internasional Indonesia ...</t>
+          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676995/komisi-xi-pfii-peluang-ri-tangkap-momentum-perpindahan-modal-global</t>
+          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/Saham-dan-oblogasi.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>ekonomi-finansial</t>
+          <t>ekonomi-bisnis</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>BUMA International Group bukukan pertumbuhan EBITDA semester I/2026</t>
+          <t>Wamen ATR: Ujian PPAT upaya berikan layanan yang baik</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Mon, 03 Aug 2026 06:17:40 +0700</t>
+          <t>Mon, 03 Aug 2026 23:05:29 +0700</t>
         </is>
       </c>
       <c r="D388" t="inlineStr"/>
       <c r="E388" t="inlineStr">
         <is>
-          <t>PT BUMA Internasional Gorup membukukan pertumbuhan EBITDA pada semester pertama 2026 (1H26) di tengah penurunan ...</t>
+          <t>Wakil Menteri Agraria dan Tata Ruang/Wakil Kepala Badan Pertanahan Nasional (Wamen ATR/Waka BPN) Ossy Dermawan ...</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5676967/buma-international-group-bukukan-pertumbuhan-ebitda-semester-i-2026</t>
+          <t>https://www.antaranews.com/berita/5678489/wamen-atr-ujian-ppat-upaya-berikan-layanan-yang-baik</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/08/02/buma.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/03/IMG_20260803_223512.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>